<commit_message>
feat: central de alarmes de calibracao anual e recarga de creditos (instrumentos e equipamentos RDC 611)
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT21"/>
+  <dimension ref="A1:AW22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -645,6 +645,21 @@
       <c r="AT1" t="inlineStr">
         <is>
           <t>peca_baixada_ref</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>tecnico_auxiliar</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>video_evidencia</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>formulario_anexo</t>
         </is>
       </c>
     </row>
@@ -767,6 +782,9 @@
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr"/>
       <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -867,6 +885,9 @@
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr"/>
       <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -967,6 +988,9 @@
       <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="inlineStr"/>
       <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1067,6 +1091,9 @@
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="inlineStr"/>
       <c r="AT5" t="inlineStr"/>
+      <c r="AU5" t="inlineStr"/>
+      <c r="AV5" t="inlineStr"/>
+      <c r="AW5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1167,6 +1194,9 @@
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="inlineStr"/>
       <c r="AT6" t="inlineStr"/>
+      <c r="AU6" t="inlineStr"/>
+      <c r="AV6" t="inlineStr"/>
+      <c r="AW6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1267,6 +1297,9 @@
       <c r="AR7" t="inlineStr"/>
       <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="inlineStr"/>
+      <c r="AU7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr"/>
+      <c r="AW7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1367,6 +1400,9 @@
       <c r="AR8" t="inlineStr"/>
       <c r="AS8" t="inlineStr"/>
       <c r="AT8" t="inlineStr"/>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr"/>
+      <c r="AW8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1467,6 +1503,9 @@
       <c r="AR9" t="inlineStr"/>
       <c r="AS9" t="inlineStr"/>
       <c r="AT9" t="inlineStr"/>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr"/>
+      <c r="AW9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1567,6 +1606,9 @@
       <c r="AR10" t="inlineStr"/>
       <c r="AS10" t="inlineStr"/>
       <c r="AT10" t="inlineStr"/>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr"/>
+      <c r="AW10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1667,6 +1709,9 @@
       <c r="AR11" t="inlineStr"/>
       <c r="AS11" t="inlineStr"/>
       <c r="AT11" t="inlineStr"/>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr"/>
+      <c r="AW11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1767,6 +1812,9 @@
       <c r="AR12" t="inlineStr"/>
       <c r="AS12" t="inlineStr"/>
       <c r="AT12" t="inlineStr"/>
+      <c r="AU12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr"/>
+      <c r="AW12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1867,6 +1915,9 @@
       <c r="AR13" t="inlineStr"/>
       <c r="AS13" t="inlineStr"/>
       <c r="AT13" t="inlineStr"/>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr"/>
+      <c r="AW13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1967,6 +2018,9 @@
       <c r="AR14" t="inlineStr"/>
       <c r="AS14" t="inlineStr"/>
       <c r="AT14" t="inlineStr"/>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr"/>
+      <c r="AW14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2083,6 +2137,9 @@
       <c r="AR15" t="inlineStr"/>
       <c r="AS15" t="inlineStr"/>
       <c r="AT15" t="inlineStr"/>
+      <c r="AU15" t="inlineStr"/>
+      <c r="AV15" t="inlineStr"/>
+      <c r="AW15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2175,6 +2232,9 @@
       <c r="AR16" t="inlineStr"/>
       <c r="AS16" t="inlineStr"/>
       <c r="AT16" t="inlineStr"/>
+      <c r="AU16" t="inlineStr"/>
+      <c r="AV16" t="inlineStr"/>
+      <c r="AW16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2303,6 +2363,9 @@
       <c r="AR17" t="inlineStr"/>
       <c r="AS17" t="inlineStr"/>
       <c r="AT17" t="inlineStr"/>
+      <c r="AU17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr"/>
+      <c r="AW17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2415,6 +2478,9 @@
       <c r="AR18" t="inlineStr"/>
       <c r="AS18" t="inlineStr"/>
       <c r="AT18" t="inlineStr"/>
+      <c r="AU18" t="inlineStr"/>
+      <c r="AV18" t="inlineStr"/>
+      <c r="AW18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2527,6 +2593,9 @@
       <c r="AR19" t="inlineStr"/>
       <c r="AS19" t="inlineStr"/>
       <c r="AT19" t="inlineStr"/>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr"/>
+      <c r="AW19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2639,6 +2708,9 @@
       <c r="AR20" t="inlineStr"/>
       <c r="AS20" t="inlineStr"/>
       <c r="AT20" t="inlineStr"/>
+      <c r="AU20" t="inlineStr"/>
+      <c r="AV20" t="inlineStr"/>
+      <c r="AW20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2775,6 +2847,176 @@
       <c r="AR21" t="inlineStr"/>
       <c r="AS21" t="inlineStr"/>
       <c r="AT21" t="inlineStr"/>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="inlineStr"/>
+      <c r="AW21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HOSPITAL SAO CARLOS</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>COMPACTO PLUS 300</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>(85) 3254-2929</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>AVENIDA PONTES VIEIRA, 2531 - DIONISIO TORRES, FOTALEZA</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>SRA. DAMARES</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>[P1 - EMERGÊNCIA MÉDICA] CHAMADO TESTE DEMONSTRATIVO EMEDONLINE: FALHA NO CONSOLE OPERACIONAL E QUEDA DE FEIXE.</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>ENERGIA: 🟢 Não foi observada  | DISJ: 🟢 Normal (Nenhum des | REBOOT: 🔄 Sim, reiniciamos e</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO - CFT</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>[EMEDONLINE] Chamado teste demonstrativo EmedOnline: Falha no console operacional e queda de feixe. | [REDE ELÉTRICA: 🟢 Não foi observada oscilação (Fornecimento normal)] [DISJUNTOR/NOBREAK: 🟢 Normal (Nenhum desarme ou alarme sonoro)] [REINICIALIZAÇÃO: 🔄 Sim, reiniciamos e o erro persistiu] [SINAIS: 🟢 Nenhum ruído ou aquecimento (Erro apenas no display)] | Solicitante: SRA. DAMARES</t>
+        </is>
+      </c>
+      <c r="W22" t="inlineStr"/>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>Não cadastrado</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr"/>
+      <c r="Z22" t="inlineStr"/>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>AVENIDA PONTES VIEIRA, 2531 - DIONISIO TORRES, FOTALEZA</t>
+        </is>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>MALETA DE CALIBRAÇÃO PADRÃO</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>CORRETIVA EMEDONLINE</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr"/>
+      <c r="AG22" t="inlineStr"/>
+      <c r="AH22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI22" t="inlineStr">
+        <is>
+          <t>CHAMADO TESTE DEMONSTRATIVO EMEDONLINE: FALHA NO CONSOLE OPERACIONAL E QUEDA DE FEIXE.</t>
+        </is>
+      </c>
+      <c r="AJ22" t="inlineStr">
+        <is>
+          <t>PARADO (INOPERANTE)</t>
+        </is>
+      </c>
+      <c r="AK22" t="inlineStr"/>
+      <c r="AL22" t="inlineStr"/>
+      <c r="AM22" t="inlineStr"/>
+      <c r="AN22" t="inlineStr"/>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>Chamado aberto via EmedOnline em 20/10/2026 18:08.</t>
+        </is>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>EM ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AQ22" t="inlineStr"/>
+      <c r="AR22" t="inlineStr"/>
+      <c r="AS22" t="inlineStr"/>
+      <c r="AT22" t="inlineStr"/>
+      <c r="AU22" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV22" t="inlineStr"/>
+      <c r="AW22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(processos): correcao na conversao de peca em teste para aplicacao definitiva (valor_os e condicao de pagamento) e normalizacao de status
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW22"/>
+  <dimension ref="A1:BA22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -662,6 +662,26 @@
           <t>formulario_anexo</t>
         </is>
       </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>data_ultima_calibracao</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>data_validade_calibracao</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>certificado_calibracao</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>requer_calibracao_anual</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -732,7 +752,11 @@
           <t>É NECESSARIO SUBSTITUIR O BOTAO DA PERA</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr"/>
       <c r="R2" t="inlineStr"/>
@@ -785,6 +809,14 @@
       <c r="AU2" t="inlineStr"/>
       <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="inlineStr"/>
+      <c r="BA2" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -836,10 +868,14 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>LEVAR PESO PARA BALANCEAR A ESTATIVA PORTA TUBO.</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr"/>
+          <t>[CONCLUÍDO - PROPOSTA APROVADA] Peça PLACA DE FONTE DE ALTA TENSÃO validada e aplicada em definitivo.</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>CONCLUÍDO</t>
+        </is>
+      </c>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr"/>
@@ -884,10 +920,22 @@
       <c r="AQ3" t="inlineStr"/>
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr">
+        <is>
+          <t>1x PLACA DE FONTE DE ALTA TENSÃO</t>
+        </is>
+      </c>
       <c r="AU3" t="inlineStr"/>
       <c r="AV3" t="inlineStr"/>
       <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="inlineStr"/>
+      <c r="BA3" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -923,7 +971,11 @@
           <t>TONY</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>5585933333333</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>NAO</t>
@@ -939,10 +991,14 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>SUBSTITUIR TECLADO DE MEMBRANA</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr"/>
+          <t>[PEÇA DE TESTE RETIRADA] SENSOR DE TEMPERATURA DEVOLVIDA AO ESTOQUE. MOTIVO: FALHA NA VERDADE ERA NO CABO DE ATERRAMENTO. PEÇA DE TESTE RETIRADA INTACTA.</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
@@ -991,6 +1047,26 @@
       <c r="AU4" t="inlineStr"/>
       <c r="AV4" t="inlineStr"/>
       <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>20/01/2026</t>
+        </is>
+      </c>
+      <c r="AY4" t="inlineStr">
+        <is>
+          <t>20/01/2027</t>
+        </is>
+      </c>
+      <c r="AZ4" t="inlineStr">
+        <is>
+          <t>LAUDO-RX-2026-55</t>
+        </is>
+      </c>
+      <c r="BA4" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -1023,7 +1099,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ANTONIO MATOS</t>
+          <t>ANTONIO</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -1045,7 +1121,11 @@
           <t>SEM PENDENCIAS APARENTES</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
@@ -1094,6 +1174,14 @@
       <c r="AU5" t="inlineStr"/>
       <c r="AV5" t="inlineStr"/>
       <c r="AW5" t="inlineStr"/>
+      <c r="AX5" t="inlineStr"/>
+      <c r="AY5" t="inlineStr"/>
+      <c r="AZ5" t="inlineStr"/>
+      <c r="BA5" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -1126,7 +1214,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>MARQUINHOS</t>
+          <t>MARCOS</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -1148,7 +1236,11 @@
           <t>SEM PENDENCIAS APARENTES</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
@@ -1197,6 +1289,14 @@
       <c r="AU6" t="inlineStr"/>
       <c r="AV6" t="inlineStr"/>
       <c r="AW6" t="inlineStr"/>
+      <c r="AX6" t="inlineStr"/>
+      <c r="AY6" t="inlineStr"/>
+      <c r="AZ6" t="inlineStr"/>
+      <c r="BA6" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -1251,7 +1351,11 @@
           <t>SEM PENDENCIAS APARENTES</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
@@ -1300,6 +1404,14 @@
       <c r="AU7" t="inlineStr"/>
       <c r="AV7" t="inlineStr"/>
       <c r="AW7" t="inlineStr"/>
+      <c r="AX7" t="inlineStr"/>
+      <c r="AY7" t="inlineStr"/>
+      <c r="AZ7" t="inlineStr"/>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -1354,7 +1466,11 @@
           <t>SEM PENDENCIAS APARENTES</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
@@ -1403,6 +1519,26 @@
       <c r="AU8" t="inlineStr"/>
       <c r="AV8" t="inlineStr"/>
       <c r="AW8" t="inlineStr"/>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>02/10/2025</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>LAUDO-RAD-2025-88</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1457,7 +1593,11 @@
           <t>SEM PENDENCIAS APARENTES</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P9" t="inlineStr"/>
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr"/>
@@ -1506,6 +1646,14 @@
       <c r="AU9" t="inlineStr"/>
       <c r="AV9" t="inlineStr"/>
       <c r="AW9" t="inlineStr"/>
+      <c r="AX9" t="inlineStr"/>
+      <c r="AY9" t="inlineStr"/>
+      <c r="AZ9" t="inlineStr"/>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1538,7 +1686,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>ANTONIO MATOS</t>
+          <t>ANTONIO</t>
         </is>
       </c>
       <c r="H10" t="inlineStr"/>
@@ -1560,7 +1708,11 @@
           <t>SEM PENDENCIAS APARENTES</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P10" t="inlineStr"/>
       <c r="Q10" t="inlineStr"/>
       <c r="R10" t="inlineStr"/>
@@ -1609,6 +1761,14 @@
       <c r="AU10" t="inlineStr"/>
       <c r="AV10" t="inlineStr"/>
       <c r="AW10" t="inlineStr"/>
+      <c r="AX10" t="inlineStr"/>
+      <c r="AY10" t="inlineStr"/>
+      <c r="AZ10" t="inlineStr"/>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1641,7 +1801,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>MARQUINHOS</t>
+          <t>MARCOS</t>
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
@@ -1663,7 +1823,11 @@
           <t>SEM PENDENCIAS APARENTES</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P11" t="inlineStr"/>
       <c r="Q11" t="inlineStr"/>
       <c r="R11" t="inlineStr"/>
@@ -1712,6 +1876,26 @@
       <c r="AU11" t="inlineStr"/>
       <c r="AV11" t="inlineStr"/>
       <c r="AW11" t="inlineStr"/>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>02/10/2025</t>
+        </is>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>02/10/2026</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>LAUDO-RAD-2025-88</t>
+        </is>
+      </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1766,7 +1950,11 @@
           <t>SEM PENDENCIAS APARENTES</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P12" t="inlineStr"/>
       <c r="Q12" t="inlineStr"/>
       <c r="R12" t="inlineStr"/>
@@ -1815,6 +2003,14 @@
       <c r="AU12" t="inlineStr"/>
       <c r="AV12" t="inlineStr"/>
       <c r="AW12" t="inlineStr"/>
+      <c r="AX12" t="inlineStr"/>
+      <c r="AY12" t="inlineStr"/>
+      <c r="AZ12" t="inlineStr"/>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1869,7 +2065,11 @@
           <t>SEM PENDENCIAS APARENTES</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P13" t="inlineStr"/>
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
@@ -1918,6 +2118,14 @@
       <c r="AU13" t="inlineStr"/>
       <c r="AV13" t="inlineStr"/>
       <c r="AW13" t="inlineStr"/>
+      <c r="AX13" t="inlineStr"/>
+      <c r="AY13" t="inlineStr"/>
+      <c r="AZ13" t="inlineStr"/>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1972,7 +2180,11 @@
           <t>SEM PENDENCIAS APARENTES</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P14" t="inlineStr"/>
       <c r="Q14" t="inlineStr"/>
       <c r="R14" t="inlineStr"/>
@@ -2021,6 +2233,26 @@
       <c r="AU14" t="inlineStr"/>
       <c r="AV14" t="inlineStr"/>
       <c r="AW14" t="inlineStr"/>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>08/11/2025</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>08/11/2026</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>LAUDO-RAD-2025-104</t>
+        </is>
+      </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -2091,7 +2323,11 @@
           <t>SOLICITAR NOBREAK</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P15" t="inlineStr"/>
       <c r="Q15" t="inlineStr"/>
       <c r="R15" t="inlineStr"/>
@@ -2140,6 +2376,26 @@
       <c r="AU15" t="inlineStr"/>
       <c r="AV15" t="inlineStr"/>
       <c r="AW15" t="inlineStr"/>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>15/03/2027</t>
+        </is>
+      </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>LAUDO-TC-2026-12</t>
+        </is>
+      </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -2186,7 +2442,11 @@
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
@@ -2235,6 +2495,14 @@
       <c r="AU16" t="inlineStr"/>
       <c r="AV16" t="inlineStr"/>
       <c r="AW16" t="inlineStr"/>
+      <c r="AX16" t="inlineStr"/>
+      <c r="AY16" t="inlineStr"/>
+      <c r="AZ16" t="inlineStr"/>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -2366,6 +2634,14 @@
       <c r="AU17" t="inlineStr"/>
       <c r="AV17" t="inlineStr"/>
       <c r="AW17" t="inlineStr"/>
+      <c r="AX17" t="inlineStr"/>
+      <c r="AY17" t="inlineStr"/>
+      <c r="AZ17" t="inlineStr"/>
+      <c r="BA17" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2398,10 +2674,14 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>A DEFINIR</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr"/>
+          <t>ARQUIMEDES</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>5585977777777</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>NÃO</t>
@@ -2481,6 +2761,14 @@
       <c r="AU18" t="inlineStr"/>
       <c r="AV18" t="inlineStr"/>
       <c r="AW18" t="inlineStr"/>
+      <c r="AX18" t="inlineStr"/>
+      <c r="AY18" t="inlineStr"/>
+      <c r="AZ18" t="inlineStr"/>
+      <c r="BA18" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -2596,6 +2884,14 @@
       <c r="AU19" t="inlineStr"/>
       <c r="AV19" t="inlineStr"/>
       <c r="AW19" t="inlineStr"/>
+      <c r="AX19" t="inlineStr"/>
+      <c r="AY19" t="inlineStr"/>
+      <c r="AZ19" t="inlineStr"/>
+      <c r="BA19" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -2711,6 +3007,14 @@
       <c r="AU20" t="inlineStr"/>
       <c r="AV20" t="inlineStr"/>
       <c r="AW20" t="inlineStr"/>
+      <c r="AX20" t="inlineStr"/>
+      <c r="AY20" t="inlineStr"/>
+      <c r="AZ20" t="inlineStr"/>
+      <c r="BA20" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -2850,6 +3154,26 @@
       <c r="AU21" t="inlineStr"/>
       <c r="AV21" t="inlineStr"/>
       <c r="AW21" t="inlineStr"/>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="AY21" t="inlineStr">
+        <is>
+          <t>15/03/2027</t>
+        </is>
+      </c>
+      <c r="AZ21" t="inlineStr">
+        <is>
+          <t>LAUDO-TC-2026-12</t>
+        </is>
+      </c>
+      <c r="BA21" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -3017,6 +3341,14 @@
       </c>
       <c r="AV22" t="inlineStr"/>
       <c r="AW22" t="inlineStr"/>
+      <c r="AX22" t="inlineStr"/>
+      <c r="AY22" t="inlineStr"/>
+      <c r="AZ22" t="inlineStr"/>
+      <c r="BA22" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(chamados): trava anti-duplicacao e debounce para impedir abertura multipla de OS por clique repetido
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA22"/>
+  <dimension ref="A1:BA25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3350,6 +3350,531 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HOSPITAL SAO CARLOS</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>COMPACTO PLUS 300</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>LEONARDO</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>(85) 3254-2929</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>AVENIDA PONTES VIEIRA, 2531 - DIONISIO TORRES, FOTALEZA</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>SRA. DAMARES</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>[P1 - EMERGÊNCIA MÉDICA] EQUIPAMENTO NAO ESTA DISPARANDO, AO TENTAR REALIZAR O EXAME O MESMO NAO GIRA O ANODO.</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Quadro / P: 🟢 Fornecimento normal (PD | Gantry &amp; M: 🟢 Gantry energizado, rota | Console de: 🟢 Console inicializa norm</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>LEONARDO - CFT</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>[EMEDONLINE - TOMOGRAFIA] Equipamento nao esta disparando, ao tentar realizar o exame o mesmo nao gira o anodo. | [Quadro / PDU / Estabilizador: 🟢 Fornecimento normal (PDU e Nobreak/Estabilizador operacionais)] [Gantry &amp; Mesa: 🟢 Gantry energizado, rotação livre e mesa movimenta normalmente] [Console de Operação: 🟢 Console inicializa normalmente e abre tela de exames] | Solicitante: SRA. DAMARES</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\FOTO_EMEDONLINE_20261020_224345_Captura de tela 2026-10-13 233530.png</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>Não cadastrado</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr"/>
+      <c r="Z23" t="inlineStr"/>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>AVENIDA PONTES VIEIRA, 2531 - DIONISIO TORRES, FOTALEZA</t>
+        </is>
+      </c>
+      <c r="AC23" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>SUGESTÃO GERAL DE ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>CORRETIVA EMEDONLINE (TOMOGRAFIA)</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr"/>
+      <c r="AG23" t="inlineStr"/>
+      <c r="AH23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI23" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTO NAO ESTA DISPARANDO, AO TENTAR REALIZAR O EXAME O MESMO NAO GIRA O ANODO.</t>
+        </is>
+      </c>
+      <c r="AJ23" t="inlineStr">
+        <is>
+          <t>PARADO (INOPERANTE)</t>
+        </is>
+      </c>
+      <c r="AK23" t="inlineStr"/>
+      <c r="AL23" t="inlineStr"/>
+      <c r="AM23" t="inlineStr"/>
+      <c r="AN23" t="inlineStr"/>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>Chamado aberto via EmedOnline (TOMOGRAFIA) em 20/10/2026 22:43.</t>
+        </is>
+      </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>EM ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AQ23" t="inlineStr"/>
+      <c r="AR23" t="inlineStr"/>
+      <c r="AS23" t="inlineStr"/>
+      <c r="AT23" t="inlineStr"/>
+      <c r="AU23" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV23" t="inlineStr"/>
+      <c r="AW23" t="inlineStr"/>
+      <c r="AX23" t="inlineStr"/>
+      <c r="AY23" t="inlineStr"/>
+      <c r="AZ23" t="inlineStr"/>
+      <c r="BA23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>24</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CLEMIR ARAIS</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>JUAZEIRO</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>DO (SALESIANO).</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>(85) 3254-2929</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>FORTALEZA - CE</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>ZELIA</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>859858585858585</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>[P2 - PROGRAMADO] - ERRO DE REINICIALIZACAO DE SCANNER, FOI REINICIADO E VOLTOU A FUNCIONAR.</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Fonte HV &amp;: 🟡 Oscilação momentânea na | Mesa, Braç: 🟢 Braço C desliza suaveme | Computador: 🟢 Software comunica norma</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO - CFT</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>[EMEDONLINE - DENSITOMETRIA] - erro de reinicializacao de scanner, foi reiniciado e voltou a funcionar. | [Fonte HV &amp; Alimentação: 🟡 Oscilação momentânea na rede elétrica] [Mesa, Braço C &amp; Shutter: 🟢 Braço C desliza suavemente sobre a mesa e shutter abre normal] [Computador &amp; Cabos HV: 🟢 Software comunica normalmente com o equipamento] | Solicitante: Zelia</t>
+        </is>
+      </c>
+      <c r="W24" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\FOTO_EMEDONLINE_20261020_233854_Captura de tela 2026-10-13 230859.png</t>
+        </is>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>Não cadastrado</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr"/>
+      <c r="Z24" t="inlineStr"/>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>859858585858585</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>Fortaleza - CE</t>
+        </is>
+      </c>
+      <c r="AC24" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>SUGESTÃO GERAL DE ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>CORRETIVA EMEDONLINE (DENSITOMETRIA)</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr"/>
+      <c r="AG24" t="inlineStr"/>
+      <c r="AH24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI24" t="inlineStr">
+        <is>
+          <t>- ERRO DE REINICIALIZACAO DE SCANNER, FOI REINICIADO E VOLTOU A FUNCIONAR.</t>
+        </is>
+      </c>
+      <c r="AJ24" t="inlineStr">
+        <is>
+          <t>OPERANDO COM FALHA</t>
+        </is>
+      </c>
+      <c r="AK24" t="inlineStr"/>
+      <c r="AL24" t="inlineStr"/>
+      <c r="AM24" t="inlineStr"/>
+      <c r="AN24" t="inlineStr"/>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>Chamado aberto via EmedOnline (DENSITOMETRIA) em 20/10/2026 23:38.</t>
+        </is>
+      </c>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>EM ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AQ24" t="inlineStr"/>
+      <c r="AR24" t="inlineStr"/>
+      <c r="AS24" t="inlineStr"/>
+      <c r="AT24" t="inlineStr"/>
+      <c r="AU24" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV24" t="inlineStr"/>
+      <c r="AW24" t="inlineStr"/>
+      <c r="AX24" t="inlineStr"/>
+      <c r="AY24" t="inlineStr"/>
+      <c r="AZ24" t="inlineStr"/>
+      <c r="BA24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>28</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CLEMIR ARAIS</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>JUAZEIRO</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>DO (SALESIANO).</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>(85) 3254-2929</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>FORTALEZA - CE</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>ZELIA</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>859858585858585</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>[P2 - PROGRAMADO] EQUIPAMENTO APRESENTANDO FALHA NA REINICIALIZACAO DO SCANNER.</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Fonte HV &amp;: ⚪ Nenhuma das opções / Nã | Mesa, Braç: ⚪ Nenhuma das opções / Ou | Computador: ⚠️ Erro de comunicação se</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO - CFT</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>[EMEDONLINE - DENSITOMETRIA] equipamento apresentando falha na reinicializacao do scanner. | [Fonte HV &amp; Alimentação: ⚪ Nenhuma das opções / Não se aplica] [Mesa, Braço C &amp; Shutter: ⚪ Nenhuma das opções / Outro comportamento] [Computador &amp; Cabos HV: ⚠️ Erro de comunicação serial/USB entre computador e mesa] | Solicitante: Zelia</t>
+        </is>
+      </c>
+      <c r="W25" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\FOTO_EMEDONLINE_20261020_234413_Captura de tela 2026-10-13 230859.png</t>
+        </is>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>Não cadastrado</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr"/>
+      <c r="Z25" t="inlineStr"/>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>859858585858585</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>Fortaleza - CE</t>
+        </is>
+      </c>
+      <c r="AC25" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>SUGESTÃO GERAL DE ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>CORRETIVA EMEDONLINE (DENSITOMETRIA)</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr"/>
+      <c r="AG25" t="inlineStr"/>
+      <c r="AH25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI25" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTO APRESENTANDO FALHA NA REINICIALIZACAO DO SCANNER.</t>
+        </is>
+      </c>
+      <c r="AJ25" t="inlineStr">
+        <is>
+          <t>OPERANDO COM FALHA</t>
+        </is>
+      </c>
+      <c r="AK25" t="inlineStr"/>
+      <c r="AL25" t="inlineStr"/>
+      <c r="AM25" t="inlineStr"/>
+      <c r="AN25" t="inlineStr"/>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>Chamado aberto via EmedOnline (DENSITOMETRIA) em 20/10/2026 23:44.</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>EM ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AQ25" t="inlineStr"/>
+      <c r="AR25" t="inlineStr"/>
+      <c r="AS25" t="inlineStr"/>
+      <c r="AT25" t="inlineStr"/>
+      <c r="AU25" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV25" t="inlineStr"/>
+      <c r="AW25" t="inlineStr"/>
+      <c r="AX25" t="inlineStr"/>
+      <c r="AY25" t="inlineStr"/>
+      <c r="AZ25" t="inlineStr"/>
+      <c r="BA25" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(estoque): correcao na extracao de codigo de pecas e baixa automatica de saldo fisico ao fechar OS
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA25"/>
+  <dimension ref="A1:BA27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3875,6 +3875,396 @@
       <c r="AZ25" t="inlineStr"/>
       <c r="BA25" t="inlineStr"/>
     </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>34</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CLINICA IMEDIATA</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ARARIPINA</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>MM SIEMENS</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>PREVENTIVA COM REPARO</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>NETTO</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>5585988888888</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>AVENIDA CENTRAL, 500 - CENTRO</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>DRA. MARIANA - BIOMÉDICA</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>(87) 98888-1234</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>[P3 - PREVENTIVA PROGRAMADA] PEDAL ESQUERDO DO COMPRESSOR COM FALHA</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>CONCLUÍDO</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>3h 30m</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Alimentação: Normal | Compressor: Ajustado | Painel: Ok</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>DRA. MARIANA ROCHA - BIOMÉDICA</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>VALFREDO V. O. NETTO - CFT 12345/CE</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>[EMEDONLINE - MAMOGRAFIA] Ajuste de pedal e calibração de rotina</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr"/>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>12.345.678/0001-90</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>56280-000</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>radiologia@imediata.com.br</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>87988881234</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>AVENIDA CENTRAL, 500 - ARARIPINA/PE</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>SUGESTÃO: AFERIÇÃO RADIOMÉTRICA &amp; FOTOCÉLULA / AEC (MULTÍMETRO 1000V)</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>PREVENTIVA / CALIBRAÇÃO (MAMOGRAFIA)</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr"/>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>FATURAMENTO 30 DIAS — R$ 380,00</t>
+        </is>
+      </c>
+      <c r="AH26" t="n">
+        <v>380</v>
+      </c>
+      <c r="AI26" t="inlineStr">
+        <is>
+          <t>PEDAL DE COMPRESSAO NAO ESTA FUNCIONANDO (PEDAL ESQUERDO)</t>
+        </is>
+      </c>
+      <c r="AJ26" t="inlineStr">
+        <is>
+          <t>OPERACIONAL COM PENDÊNCIA (AGUARDA PREVENTIVA)</t>
+        </is>
+      </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>Microswitch com resistência de contato de 45 Ohms (queimado)</t>
+        </is>
+      </c>
+      <c r="AL26" t="inlineStr">
+        <is>
+          <t>Desgaste mecânico do microswitch do pedal de compressão esquerdo</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>Substituído microswitch por peça nova original Siemens (PEC-006). Realizada calibração de força do compressor com célula de carga aferida: 15 daN a 20 daN conforme protocolo. Validação de resolução espacial e contraste com Phantom de Mamografia aprovada.</t>
+        </is>
+      </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>Força de compressão: 18 daN | Espessura acrílica: 45mm | kVp medido: 28 kV | Reprodutibilidade: CV &lt; 0.02</t>
+        </is>
+      </c>
+      <c r="AO26" t="inlineStr">
+        <is>
+          <t>Equipamento 100% liberado para atendimento clínico de rotina.</t>
+        </is>
+      </c>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>LIBERADO PARA USO NORMAL</t>
+        </is>
+      </c>
+      <c r="AQ26" t="inlineStr"/>
+      <c r="AR26" t="inlineStr"/>
+      <c r="AS26" t="inlineStr"/>
+      <c r="AT26" t="inlineStr"/>
+      <c r="AU26" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV26" t="inlineStr"/>
+      <c r="AW26" t="inlineStr"/>
+      <c r="AX26" t="inlineStr"/>
+      <c r="AY26" t="inlineStr"/>
+      <c r="AZ26" t="inlineStr"/>
+      <c r="BA26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>35</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>CLINICA IMEDIATA</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>ARARIPINA</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>(85) 3254-2929</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>FORTALEZA - CE</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>PEDRO</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>34684651654</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>[P1 - EMERGÊNCIA MÉDICA] EQUIPAMENTO NAO LIGA</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Fonte HV &amp;: 🟡 Oscilação momentânea na | Mesa, Braç: ⚪ Nenhuma das opções / Ou | Computador: ⚪ Nenhuma das opções / Nã</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr"/>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO - CFT</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>[EMEDONLINE - DENSITOMETRIA] equipamento nao liga | [Fonte HV &amp; Alimentação: 🟡 Oscilação momentânea na rede elétrica] [Mesa, Braço C &amp; Shutter: ⚪ Nenhuma das opções / Outro comportamento] [Computador &amp; Cabos HV: ⚪ Nenhuma das opções / Não se aplica] | Solicitante: pedro</t>
+        </is>
+      </c>
+      <c r="W27" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\FOTO_EMEDONLINE_20261021_004453_Captura de tela 2026-10-13 230859.png</t>
+        </is>
+      </c>
+      <c r="X27" t="inlineStr">
+        <is>
+          <t>Não cadastrado</t>
+        </is>
+      </c>
+      <c r="Y27" t="inlineStr"/>
+      <c r="Z27" t="inlineStr"/>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>34684651654</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
+        <is>
+          <t>Fortaleza - CE</t>
+        </is>
+      </c>
+      <c r="AC27" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD27" t="inlineStr">
+        <is>
+          <t>SUGESTÃO: CALIBRAÇÃO &amp; MANUTENÇÃO EM DENSITOMETRIA ÓSSEA</t>
+        </is>
+      </c>
+      <c r="AE27" t="inlineStr">
+        <is>
+          <t>CORRETIVA EMEDONLINE (DENSITOMETRIA)</t>
+        </is>
+      </c>
+      <c r="AF27" t="inlineStr"/>
+      <c r="AG27" t="inlineStr"/>
+      <c r="AH27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI27" t="inlineStr">
+        <is>
+          <t>EQUIPAMENTO NAO LIGA</t>
+        </is>
+      </c>
+      <c r="AJ27" t="inlineStr">
+        <is>
+          <t>PARADO (INOPERANTE)</t>
+        </is>
+      </c>
+      <c r="AK27" t="inlineStr"/>
+      <c r="AL27" t="inlineStr"/>
+      <c r="AM27" t="inlineStr"/>
+      <c r="AN27" t="inlineStr"/>
+      <c r="AO27" t="inlineStr">
+        <is>
+          <t>Chamado aberto via EmedOnline (DENSITOMETRIA) em 21/10/2026 00:44.</t>
+        </is>
+      </c>
+      <c r="AP27" t="inlineStr">
+        <is>
+          <t>EM ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AQ27" t="inlineStr"/>
+      <c r="AR27" t="inlineStr"/>
+      <c r="AS27" t="inlineStr"/>
+      <c r="AT27" t="inlineStr"/>
+      <c r="AU27" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV27" t="inlineStr"/>
+      <c r="AW27" t="inlineStr"/>
+      <c r="AX27" t="inlineStr"/>
+      <c r="AY27" t="inlineStr"/>
+      <c r="AZ27" t="inlineStr"/>
+      <c r="BA27" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: auditoria integral 100% concluida, ITs de manuais tecnicos e geracao QR offline
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -1099,7 +1099,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ANTONIO</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H5" t="inlineStr"/>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>MARCOS</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H6" t="inlineStr"/>
@@ -1329,7 +1329,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>GABRIEL</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H7" t="inlineStr"/>
@@ -1444,7 +1444,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>PAULO</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -1571,7 +1571,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>YASMIM</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -2801,7 +2801,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>A DEFINIR</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H19" t="inlineStr"/>
@@ -2924,7 +2924,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>A DEFINIR</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H20" t="inlineStr"/>

</xml_diff>

<commit_message>
feat: link avaliacao Google nas OS, correcao QR celular com base url dinamica e rotulos manuais
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA27"/>
+  <dimension ref="A1:BA29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -968,17 +968,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>TONY</t>
+          <t>ANTONIO</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>5585933333333</t>
+          <t>85996199711</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1017,7 +1017,11 @@
           <t>CONTRATO</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>LEVA TERROMETRO PARA VERIFICA ATERRAMENTO</t>
+        </is>
+      </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
@@ -1099,10 +1103,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>NETTO</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr"/>
+          <t>ARQUIMEDES</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>5585977777777</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>NAO</t>
@@ -4265,6 +4273,352 @@
       <c r="AZ27" t="inlineStr"/>
       <c r="BA27" t="inlineStr"/>
     </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>39</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HOSPITAL SAO CARLOS</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>COMPACTO PLUS 300</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>LEONARDO</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>(85) 3254-2929</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>AVENIDA PONTES VIEIRA, 2531 - DIONISIO TORRES, FOTALEZA</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>SRA. DAMARES</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>[P1 - EMERGÊNCIA MÉDICA] PERA NAO ESTA DISPARANDO</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Alimentaçã: ⚪ Nenhuma das opções / Nã | Estativa &amp;: ⚪ Nenhuma das opções / Ou | Botão &amp; Re: ⚪ Nenhuma das opções / Nã</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr"/>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>LEONARDO - CFT</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>[EMEDONLINE - RAIO-X] pera nao esta disparando | [Alimentação Elétrica: ⚪ Nenhuma das opções / Não se aplica] [Estativa &amp; Eletrofreio: ⚪ Nenhuma das opções / Outro comportamento] [Botão &amp; Resposta Sonora: ⚪ Nenhuma das opções / Não se aplica] | Solicitante: SRA. DAMARES</t>
+        </is>
+      </c>
+      <c r="W28" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\FOTO_EMEDONLINE_20261021_094417_IMG_20260423_094025_114.jpg</t>
+        </is>
+      </c>
+      <c r="X28" t="inlineStr">
+        <is>
+          <t>Não cadastrado</t>
+        </is>
+      </c>
+      <c r="Y28" t="inlineStr"/>
+      <c r="Z28" t="inlineStr"/>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
+      </c>
+      <c r="AB28" t="inlineStr">
+        <is>
+          <t>AVENIDA PONTES VIEIRA, 2531 - DIONISIO TORRES, FOTALEZA</t>
+        </is>
+      </c>
+      <c r="AC28" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD28" t="inlineStr">
+        <is>
+          <t>SUGESTÃO GERAL DE ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AE28" t="inlineStr">
+        <is>
+          <t>CORRETIVA EMEDONLINE (RAIO-X)</t>
+        </is>
+      </c>
+      <c r="AF28" t="inlineStr"/>
+      <c r="AG28" t="inlineStr"/>
+      <c r="AH28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI28" t="inlineStr">
+        <is>
+          <t>PERA NAO ESTA DISPARANDO</t>
+        </is>
+      </c>
+      <c r="AJ28" t="inlineStr">
+        <is>
+          <t>PARADO (INOPERANTE)</t>
+        </is>
+      </c>
+      <c r="AK28" t="inlineStr"/>
+      <c r="AL28" t="inlineStr"/>
+      <c r="AM28" t="inlineStr"/>
+      <c r="AN28" t="inlineStr"/>
+      <c r="AO28" t="inlineStr">
+        <is>
+          <t>Chamado aberto via EmedOnline (RAIO-X) em 21/10/2026 09:44.</t>
+        </is>
+      </c>
+      <c r="AP28" t="inlineStr">
+        <is>
+          <t>EM ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AQ28" t="inlineStr"/>
+      <c r="AR28" t="inlineStr"/>
+      <c r="AS28" t="inlineStr"/>
+      <c r="AT28" t="inlineStr"/>
+      <c r="AU28" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV28" t="inlineStr"/>
+      <c r="AW28" t="inlineStr"/>
+      <c r="AX28" t="inlineStr"/>
+      <c r="AY28" t="inlineStr"/>
+      <c r="AZ28" t="inlineStr"/>
+      <c r="BA28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>40</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>CLEMIR ARAIS</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>JUAZEIRO</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>MM (PATIO).</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>(85) 3254-2929</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>FORTALEZA - CE</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>ZELIA</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>8598598712165</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>[P1 - EMERGÊNCIA MÉDICA] PEDAL DE COMPRESSO ESQUERDO NAO FUNCIONA</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Quadro de : ⚪ Nenhuma das opções / Nã | Gantry &amp; C: ⚪ Nenhuma das opções / Ou | Painel &amp; B: ⚪ Nenhuma das opções / Nã</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr"/>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO - CFT</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>[EMEDONLINE - MAMOGRAFIA] pedal de compresso esquerdo nao funciona | [Quadro de Força: ⚪ Nenhuma das opções / Não se aplica] [Gantry &amp; Compressor: ⚪ Nenhuma das opções / Outro comportamento] [Painel &amp; Biombo: ⚪ Nenhuma das opções / Não se aplica] | Solicitante: zelia</t>
+        </is>
+      </c>
+      <c r="W29" t="inlineStr"/>
+      <c r="X29" t="inlineStr">
+        <is>
+          <t>Não cadastrado</t>
+        </is>
+      </c>
+      <c r="Y29" t="inlineStr"/>
+      <c r="Z29" t="inlineStr"/>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>8598598712165</t>
+        </is>
+      </c>
+      <c r="AB29" t="inlineStr">
+        <is>
+          <t>Fortaleza - CE</t>
+        </is>
+      </c>
+      <c r="AC29" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD29" t="inlineStr">
+        <is>
+          <t>SUGESTÃO: AFERIÇÃO RADIOMÉTRICA &amp; FOTOCÉLULA / AEC (MULTÍMETRO 1000V)</t>
+        </is>
+      </c>
+      <c r="AE29" t="inlineStr">
+        <is>
+          <t>CORRETIVA EMEDONLINE (MAMOGRAFIA)</t>
+        </is>
+      </c>
+      <c r="AF29" t="inlineStr"/>
+      <c r="AG29" t="inlineStr"/>
+      <c r="AH29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI29" t="inlineStr">
+        <is>
+          <t>PEDAL DE COMPRESSO ESQUERDO NAO FUNCIONA</t>
+        </is>
+      </c>
+      <c r="AJ29" t="inlineStr">
+        <is>
+          <t>PARADO (INOPERANTE)</t>
+        </is>
+      </c>
+      <c r="AK29" t="inlineStr"/>
+      <c r="AL29" t="inlineStr"/>
+      <c r="AM29" t="inlineStr"/>
+      <c r="AN29" t="inlineStr"/>
+      <c r="AO29" t="inlineStr">
+        <is>
+          <t>Chamado aberto via EmedOnline (MAMOGRAFIA) em 21/10/2026 13:59.</t>
+        </is>
+      </c>
+      <c r="AP29" t="inlineStr">
+        <is>
+          <t>EM ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AQ29" t="inlineStr"/>
+      <c r="AR29" t="inlineStr"/>
+      <c r="AS29" t="inlineStr"/>
+      <c r="AT29" t="inlineStr"/>
+      <c r="AU29" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV29" t="inlineStr"/>
+      <c r="AW29" t="inlineStr"/>
+      <c r="AX29" t="inlineStr"/>
+      <c r="AY29" t="inlineStr"/>
+      <c r="AZ29" t="inlineStr"/>
+      <c r="BA29" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: triagem cirurgica de defeitos, demanda automatica almoxarifado no fechamento e mural tv de operacoes
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -1103,7 +1103,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>ARQUIMEDES</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -3389,7 +3389,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>LEONARDO</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">

</xml_diff>

<commit_message>
feat(v21): remover criogenia/helio, padronizar razao social para Diagnostico por Imagem, timbrado oficial em todas as 4 paginas da pre-instalacao Lotus HF500M
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA29"/>
+  <dimension ref="A1:BA35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -719,7 +719,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>5585911111111</t>
+          <t>85996199711</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -749,26 +749,60 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>É NECESSARIO SUBSTITUIR O BOTAO DA PERA</t>
+          <t>[CONCLUÍDO COM PENDÊNCIA: PROGRAMADA] BOTAO ANTIVANDALIMO 22MM | REALIZADO SUBSTITUIÇÃO DO BOTÃO DO HANDSWITCH (PERA).
+- REALIZADO SUBSTITUIÇÃO DA GRAXA ISOLANTE DOS CONECTORES DO CABO FEDERAL DO ANODO E CATODO.
+- REALIZADO TESTES OPERACIONAIS DE FUNCIONAMENTO.
+- REALIZADO ACOMPANHAMENTO DE EXAMES COM PACIENTES OK | [DIAGNÓSTICO: REALIZADO SUBSTITUIÇÃO DO BOTÃO DO HANDSWITCH (PERA).
+- REALIZADO SUBSTITUIÇÃO DA GRAXA ISOLANTE DOS CONECTORES DO CABO FEDERAL DO ANODO E CATODO.
+- REALIZADO TESTES OPERACIONAIS DE FUNCIONAMENTO.
+- REALIZADO ACOMPANHAMENTO DE EXAMES COM PACIENTES OK] | [FATURAMENTO BOLETO BANCÁRIO (VALOR INTEGRAL) — VALOR FINAL: R$ 0.00]</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>ATIVO</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
+          <t>CONCLUÍDO</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>22/10/2026 14:22</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>22/10/2026 14:22</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>0 min</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>LIMPEZA TÉCNICA INTERNA/EXTERNA, LUBRIFICAÇÃO DE GUIAS E ROLAMENTOS, TESTE FUNCIONAL COM OPERADOR LOCAL, INSPEÇÃO DE CABOS, CONECTORES E ATERRAMENTO, VERIFICAÇÃO DE TRAVAS E SEGURANÇA MECÂNICA</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>SRA. DAMARES</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>ANTONIO - TÉCNICO</t>
+        </is>
+      </c>
       <c r="V2" t="inlineStr"/>
       <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
+      </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr">
         <is>
@@ -777,24 +811,54 @@
       </c>
       <c r="AD2" t="inlineStr">
         <is>
-          <t>BOTAO ANTIVANDALIMO 22MM</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr"/>
+          <t>[PROGRAMADA] BOTAO ANTIVANDALIMO 22MM</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>GERAL / CORRETIVA</t>
+        </is>
+      </c>
       <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>FATURAMENTO 28 DDL</t>
+        </is>
+      </c>
       <c r="AH2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AI2" t="inlineStr"/>
+        <v>18500</v>
+      </c>
+      <c r="AI2" t="inlineStr">
+        <is>
+          <t>É NECESSARIO SUBSTITUIR O BOTAO DA PERA</t>
+        </is>
+      </c>
       <c r="AJ2" t="inlineStr">
         <is>
           <t>OPERACIONAL</t>
         </is>
       </c>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr">
+        <is>
+          <t>REALIZADO SUBSTITUIÇÃO DO BOTÃO DO HANDSWITCH (PERA).
+- REALIZADO SUBSTITUIÇÃO DA GRAXA ISOLANTE DOS CONECTORES DO CABO FEDERAL DO ANODO E CATODO.
+- REALIZADO TESTES OPERACIONAIS DE FUNCIONAMENTO.
+- REALIZADO ACOMPANHAMENTO DE EXAMES COM PACIENTES OK</t>
+        </is>
+      </c>
+      <c r="AL2" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO PREVENTIVA PROGRAMADA (SEM FALHA)</t>
+        </is>
+      </c>
+      <c r="AM2" t="inlineStr">
+        <is>
+          <t>REALIZADO SUBSTITUIÇÃO DO BOTÃO DO HANDSWITCH (PERA).
+- REALIZADO SUBSTITUIÇÃO DA GRAXA ISOLANTE DOS CONECTORES DO CABO FEDERAL DO ANODO E CATODO.
+- REALIZADO TESTES OPERACIONAIS DE FUNCIONAMENTO.
+- REALIZADO ACOMPANHAMENTO DE EXAMES COM PACIENTES OK</t>
+        </is>
+      </c>
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr">
@@ -968,7 +1032,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>ANTONIO</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -991,7 +1055,7 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>[PEÇA DE TESTE RETIRADA] SENSOR DE TEMPERATURA DEVOLVIDA AO ESTOQUE. MOTIVO: FALHA NA VERDADE ERA NO CABO DE ATERRAMENTO. PEÇA DE TESTE RETIRADA INTACTA.</t>
+          <t>[CONCLUÍDO - GERAL] Sem pendências restantes.</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -999,14 +1063,42 @@
           <t>ATIVO</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
-      <c r="Q4" t="inlineStr"/>
-      <c r="R4" t="inlineStr"/>
-      <c r="S4" t="inlineStr"/>
-      <c r="T4" t="inlineStr"/>
-      <c r="U4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>25/10/2026 23:09</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>25/10/2026 23:09</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>0 min</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>LIMPEZA TÉCNICA, TESTE FUNCIONAL COM OPERADOR, INSPEÇÃO DE CABOS E SEGURANÇA</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>DR ELIEZER</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>NETTO - TÉCNICO CFT</t>
+        </is>
+      </c>
       <c r="V4" t="inlineStr"/>
-      <c r="W4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\ANTES_OS3_20261025_230949.jpg</t>
+        </is>
+      </c>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr"/>
       <c r="Z4" t="inlineStr"/>
@@ -1017,37 +1109,73 @@
           <t>CONTRATO</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
-        <is>
-          <t>LEVA TERROMETRO PARA VERIFICA ATERRAMENTO</t>
-        </is>
-      </c>
-      <c r="AE4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
       <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>FATURAMENTO BOLETO BANCÁRIO (VALOR INTEGRAL) — VALOR FINAL: R$ 0.00</t>
+        </is>
+      </c>
       <c r="AH4" t="n">
         <v>0</v>
       </c>
-      <c r="AI4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>- EQUIPAMENTO NÃO ESTÁ DISPARANDO.</t>
+        </is>
+      </c>
       <c r="AJ4" t="inlineStr">
         <is>
           <t>OPERACIONAL</t>
         </is>
       </c>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr">
+        <is>
+          <t>- CABO E BOTAO DA PERA DANIFICADO.</t>
+        </is>
+      </c>
+      <c r="AL4" t="inlineStr">
+        <is>
+          <t>DESGASTE NATURAL</t>
+        </is>
+      </c>
+      <c r="AM4" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO PREVENTIVA E AFERIÇÃO RADIOMÉTRICA EM EQUIPAMENTO DE RAIOS-X. AFERIÇÃO DE KVP, MA E TEMPO DE DISPARO COM MULTÍMETRO RADIOMÉTRICO HOMOLOGADO. TESTE DE REPETIBILIDADE, LINEARIDADE E RENDIMENTO DO TUBO. INSPEÇÃO DA ISOLAÇÃO DOS CABOS DE ALTA TENSÃO E NÍVEL DE ÓLEO DO TANQUE GERADOR. EQUIPAMENTO LIBERADO. | [PEÇA MANUAL: 1x CABO SPIRAL E BOTÃO ANTI VANDALISMO]</t>
+        </is>
+      </c>
+      <c r="AN4" t="inlineStr">
+        <is>
+          <t>- VERIFICADO RESISTÊNCIA DO CONTATO DO BOTÃO E TESTES DAS VIAS DO CABO SPIRAL</t>
+        </is>
+      </c>
       <c r="AO4" t="inlineStr"/>
       <c r="AP4" t="inlineStr">
         <is>
           <t>LIBERADO PARA USO NORMAL</t>
         </is>
       </c>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\DEPOIS_OS3_20261025_230949.jpg</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAUAAAABuCAYAAABWQcpYAAAKn0lEQVR4AeydW44kRxWGM4axQN0tGaYb8Qji0dXABkCwBdYBD+wAswfYh5cAggUgmPYbCL8hMWNZqGcE9kynz59V0YqKzrpkVV7i8rXqdGZWZkSc+E71p8iq8vhZww8EIACBSgkgwEoLz7QhAIGmQYC8CiAAgWoJVC3AaqvOxCEAgY4AAuww8AsCEKiRAAKsserMGQIQ6AggwA5Dhb+YMgQgwIcgvAYgAIF6CbACrLf2zBwC1RNAgNW/BGoEwJwhsCaAANcc+A0BCFRIAAFWWHSmDAEIrAkgwDUHfkOgFgLMMyCAAAMY7EIAAnURQIB11ZvZQgACAQEEGMBgFwIQKJtAPDsEGBPhGAIQqIYAAqym1EwUAhCICSDAmAjHEIBANQSqEmA1VWWiEIDAUQQQ4FGYuAgCECiRAAIssarMCQIQOIoAAjwKUwEXzTCFixcfPVxer9oZhmIICIxCAAGOgpFORMDZj7YSobYEBFIngABTr1Am+YUrv7eff8rrKpO61Z4mL9TaXwFVzJ9JQqCfAALs58KzEIBABQQQYAVFZooQgEA/AQTYz4VnITAqgaub24/1Pqli1I4Pd8YVewggwD1wOHUcgfBT39Z+jmtV11WG5bd1zTiP2SLAPOqUTZZ8Avy0VLb6+6N/1jn3O7/PdnkCCHD5GmSfgbOf7Ccx0QQkP1v9/VzdG6Y/3b96+bH2iXkIHBoFAR4ixHkInEjg8mb1Gy8/6+ILk98vbMsjIQIIMKFikEphBNrm8X2/N6/vvlPY7IqYDgIsooxMIjUCuvW1nL5t0ejWV1siPQJFCzA93GRUAwHJz9/6Sn7c+qZbdQSYbm2yy8z+6PmXYKxqxqH70MN2G+QnCukGAky3NllkFn4HkK/ANI1Wf75wWv35fbZpEkCAadbl/Kxm6sH+yN1MQyU/jH3q+1e/+jMu+soLn/omXjUEmHiBSC8jAm3zE58tt76eRNpbBJh2fcguEwKX16t/+VTds+YPfp9t2gQQYNr1IbuTCMzbaCO/729G/ez+P3e/3uyzSZwAAky8QKSXNoGr765+bxk+yu/N67sf2DGPTAggwEwKRZppEmgfml/5zJCfJ5HPFgHmU6ukM7VPP6v7DuDm1tfX5TO/s/CW4QcQQIADYHHpNoHwO4DbZ8o/2siPW9/MS40AMy8g6S9GwMuv4dZ3sRqcPTACPBshHYhATf8VyGb1p2k3fOWlw5DMr6GJIMChxLi+agIb+fnVH195yfzVgAAzLyDpz0eAr7zMx3qukRDgXKQZJ3sCfOUl+xI+mUBRAnwyO56AwEgENre+vje+8uJJZL5FgJkXkPSnJ3B5s/q3jfL4vh+f+hqNQh4IsJBCMo1pCFxd337RtM33fO/Iz5MoY4sAy6hj01QyD335WmG3pO0xcQ4Wya9t2g99H865T/w+2zIIIMAy6rj4LCSlqZJQ3woJzyTUPY4dS218HNtG1/XJ7/7Vy1/qHFEOAQRYTi2LmomEp5C8OuPZr3MnqL4Uh/qJ5Nfa0J8gv0PU8jyPAPOsWxJZj/1ff0h4CknKpNM94onqH12w9+HcdtztPI7b61j9K7QfRyw/G+cZ8osplXOMAMup5aIzka1OTWCI9IZK1wTWybEvt1iCffLra8dz5RBAgOXUMruZhOKLkw9XekOlF/elYy9CbXXsw0sQ+XkidW0RYF31Hn22EpXvVELz+4e2Ek+8alRfEpRiDOntykH9h+eUS/Bpb2vnc/q7CKfC/kACFHogMC7fJjBUVJKkhLPdS6N/UsoN7SvuY8ixSc71XI/8eqCU/BQCLLm6M88tXtGFw3vxxddIRIrw2oX2kd9C4JccFgEuSb+QsXXrum8qWvHF4lObpcR3dbP6s3IKc7Zc+FsIgWSyf26aFP1cgrTfIhCLJT7WxSabWW93NaYPya9tm5/6Y7Z1E0CAddd/lNnH793pdlcRy2/JVZ8menmz+h/yEwnCE0CAngTbswhIbr4D3e4q/LG2S676NL7k17TNN7WvcK75i7ZE3QSyFmDdpUtr9vEq0GcnMUp+/njurW55u5VoID/lw0pw7kqkOR4CTLMuRWQl+e0S4xwTlPy2ROea/0t+nRCDBPRccMhuRQQQYEXFnnKqsVSmHOuYvi2fL5/I79Xdt+z5NmwvSYfH7NdFAAHmWu+E8o6l4lNz9qMPQ/zx1Nur69u/KReFjfWBRfdw9n7fmx3yW3KF2iXHr0UJIMBF8ec/+EY2jxPRikrhn3D24/en2nrxtU37o3gMZ/K7f3X3s748kV9Mq75jBFhfzUeb8S6pxGKJrxsjAS899d0rvsb9Xe/t9clPz8c5jpETfeRHAAHmV7MkMpZ4wkRiqeg4PB9fH54bsr8W38re3utZ7W2kp7HvX7/8sW6/43F1bsh4XFs2AQRYdn1Pnt3Fi9VXCgmkL+KO/TUX17dvfLSNexte568Jn9u3f3Vz+w8fvu3e1Z5Jz/en6539+GNtkZ8oECEBBBjSqHRfolNIGj6ca54rhiJxTXsRRl97P8ahrb2X+EMfcT8uWu358xcvPnpQv/5YW+tD/9CB0z4BgZAAAgxpVLR/8WL1TqJQSHSKHKbvNuLTLa7P92IjvfVcbCb+hG216ivs/T6bFY+xCCDAsUhm0o8koTBNfGNXyvYG2zuF5KHQCiq+Vs/vC93++rC2/7UY8tD/iOifzrkuwnG8+CQ9xXouzsWdK2e1i5/nGAIhAQQY0ih8X7KIp2iie2/xTrLw8fbzuw8UulZtnP1o34eu8/u7tm9fv7z0Ydd/aNH9vzm03dUmeN6ZwB5vf5VDHJZS9wjadLvWrrvdZdXX4eDXAQII8ACgEk7bSum9BBLOxaT3XjIy0T23ePzSsL/G2kz2XprGVUhWfrxztupH/SkQ3zkk0287doYIcGyiifVnIntvS6WtOq9Fcfd8V6rW5sHabN1Wrtt8utXPrvbHPi9Zqd8wjmkr4Sl8O/VzTDuugUBMYNQXdNw5x8sS0KrPRLZVY0ljX1abNk/kt6/NmOeU36GQ8BRjjktfdRLY+uOoE0F5s7YVXM8tb/sgseyarbWZ7JZ315g8D4GlCWQlwKVh5TJ+36rPVkw7P/XdteqzNrw+cik6eZ5EgBf4SdjSbSSZhdkNXfWp7b42Ok9AoBQCCLCUSto8jpGfv9XVtbZS3Hqvz3+wYF3xgEAVBBBgLmUemGe4ipP0FH3SU7defNzyigZREwEEWEi1JbdwKjr2oZWeIjyvfcQnCkTNBBBgZdX30tMKkRVfZcVnuk8IIMAnSPJ7Qiu9fVlLeop8pbdvdpyDwOkEEODp7JJpKbmFIdGFoZWeIpmESQQCiRBAgIkU4pw0JLcwzumLthCoiQACrKnazDVHAuQ8IQEEOCFcuoYABNImgADTrg/ZQQACExJAgBPCpWsIQOA8AlO3RoBTE6Z/CEAgWQIIMNnSkBgEIDA1AQQ4NWH6hwAEkiWQtACTpUZiEIBAEQQQYBFlZBIQgMApBBDgKdRoAwEIFEEAAaZaRvKCAAQmJ4AAJ0fMABCAQKoEEGCqlSEvCEBgcgIIcHLEDDCcAC0gMA8BBDgPZ0aBAAQSJIAAEywKKUEAAvMQQIDzcGYUCBxLgOtmJIAAZ4TNUBCAQFoEvgYAAP//f2lRSwAAAAZJREFUAwAhmVcZzb9DGQAAAABJRU5ErkJggg==</t>
+        </is>
+      </c>
       <c r="AS4" t="inlineStr"/>
-      <c r="AT4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>1x CABO SPIRAL E BOTÃO ANTI VANDALISMO</t>
+        </is>
+      </c>
       <c r="AU4" t="inlineStr"/>
       <c r="AV4" t="inlineStr"/>
       <c r="AW4" t="inlineStr"/>
@@ -1340,10 +1468,14 @@
           <t>NETTO</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>85999150273</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1455,10 +1587,14 @@
           <t>NETTO</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>85999150273</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1582,10 +1718,14 @@
           <t>NETTO</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>85999150273</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1606,9 +1746,21 @@
           <t>ATIVO</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>22/10/2026 17:31</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>22/10/2026 17:31</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>0 min</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr"/>
       <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr"/>
@@ -1694,13 +1846,17 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>ANTONIO</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr"/>
+          <t>NETTO</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>85999150273</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1809,13 +1965,17 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>MARCOS</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr"/>
+          <t>NETTO</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>85999150273</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -2429,13 +2589,21 @@
           <t>TC CT/E</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>ARQUIMEDES</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>5585977777777</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -2446,21 +2614,37 @@
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>SEDE EMED</t>
+        </is>
+      </c>
       <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>[CONCLUÍDO - GERAL / CORRETIVA] MANUTENÇÃO E REVISÃO TÉCNICA EXECUTADA CONFORME PROTOCOLO EMED. | [CORTESIA / COBERTO POR CONTRATO MENSAL — VALOR FINAL: R$ 0.00]</t>
+        </is>
+      </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>ATIVO</t>
+          <t>CONCLUÍDO</t>
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
       <c r="Q16" t="inlineStr"/>
       <c r="R16" t="inlineStr"/>
       <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL DO SETOR / HOSPITAL</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>ARQUIMEDES - TÉCNICO</t>
+        </is>
+      </c>
       <c r="V16" t="inlineStr"/>
       <c r="W16" t="inlineStr"/>
       <c r="X16" t="inlineStr"/>
@@ -2474,9 +2658,17 @@
         </is>
       </c>
       <c r="AD16" t="inlineStr"/>
-      <c r="AE16" t="inlineStr"/>
+      <c r="AE16" t="inlineStr">
+        <is>
+          <t>GERAL / CORRETIVA</t>
+        </is>
+      </c>
       <c r="AF16" t="inlineStr"/>
-      <c r="AG16" t="inlineStr"/>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>CORTESIA / COBERTO POR CONTRATO MENSAL — VALOR FINAL: R$ 0.00</t>
+        </is>
+      </c>
       <c r="AH16" t="n">
         <v>0</v>
       </c>
@@ -2487,8 +2679,16 @@
         </is>
       </c>
       <c r="AK16" t="inlineStr"/>
-      <c r="AL16" t="inlineStr"/>
-      <c r="AM16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO PREVENTIVA PROGRAMADA (SEM FALHA)</t>
+        </is>
+      </c>
+      <c r="AM16" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E REVISÃO TÉCNICA EXECUTADA CONFORME PROTOCOLO EMED.</t>
+        </is>
+      </c>
       <c r="AN16" t="inlineStr"/>
       <c r="AO16" t="inlineStr"/>
       <c r="AP16" t="inlineStr">
@@ -2497,7 +2697,11 @@
         </is>
       </c>
       <c r="AQ16" t="inlineStr"/>
-      <c r="AR16" t="inlineStr"/>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAggAAACbCAYAAAAHkWOnAAAQAElEQVR4AeydTZJkyVHHM2dGQsYCSWbs6WrW4gRgEjeAE7BgegULOAFwAljAqltm3ABuIGFwArSf6gtgSJhhhmxanfgvqzzLX1S8r8z3ERH5H0vvF9/h/vOX4V4vs2q+OOg/ERABERCBTQh8/fj4M5NTEOo/2WRzbSICMwkoQZgJTMNFQAREYC4BSwh+YnKyeTEZ+LsPDw9/bPJza9dLBBYmcPtyShBuZ6gVREAERKCXgCUGP7NOxC7nFwkBicHfnmv6RwQKJaAEoVDHSC0REIG6CVhioKcGdbtwV+1L2FwJQglekA4iIAJNEbDkgKcDemrQlFfvzxglCPfnc1ksAiKwEgFLDHhqQGLwN2ELfdcgwLiPYhtWKkFow4+yQgREYGcClhz4UwP/IqK+a7CzT7T9bQSUINzGT7NFQATunIAlBnpq0Ng9IHOeCChBeOKgf0VABERgNgFLDvTUYDY1TaiFgBKEWjwlPUVABIohYImBnhoU441UEdWXIqAEYSmSWkcEROAuCFhyoKcGd+FpGakEQfeACIiACEwgYImBnhpM4HTrEM0vh4AShHJ8IU1EQAQKJGCJwV+Z/LOpxq8v6jcUDIRe90FACcJ9+FlWioAIzCRgSQGJwX/btL83+TMTf+nvGjiJV1c1tERACUJL3pQtIiACNxNIEoMfhAV/aWX9PxQMgl73QUAJwn34WVaKgAiMEBhJDP76w8PDD03440cjK9XbLc1FIBJQghBpqHw1ATtcTy5//vj4+eqFNFEENiZg9238KCF9YuCJwT9srJa2E4HdCShB2N0F9StgB+wpWnE8HI5p20H/iUBhBOwebSwxKAyw1KmegBKE6l24rwF2yHaSg6gNfUhsU1kE9iZg9+TPTbhv+fKhnhjs7RDtXywBJQjFuqY+xezzWXt48Frv58P4dYdaRGAjAnYPnp8W2JXE4MfJtv/GvWvCdwx2+ygh0UlVEdidgBKE3V1QrwLPh23HADtkj0hstBPZXrFFZRHYhoDdo+fEwHbre1rA/ep/28CG6SUCIuAElCA4CV1nEbCDtxP006SAustPHx50n82iq8G3ErD7cywxWPhpwa0aa74IlEdAB3d5PileIzt8B5OD4g2Qgs0SsHtTiUGz3pVhWxNQgrA18cr3swO4kxxYxV6VGyX1qydg9+VNiUH1AGSACKxAQAnCClBbXTL39w308UGr3q7DLksM9BsJdbhKWlZIQAlChU7bS+Xj4WCvw+U/vmNwqaggAhsRsKTg/LTArjy9+vHh0NlYv5HQwaGKCFxPQAnC9ezuaubzYXyxWcnBBYUKGxH4+ptv/vHdx4/f2na530jwxEC/kWCA9BKBJQgoQViCYuNrKDlo3ME7mze2/SUxOB7/4nQ6fRXG8z9P8j+FrMQggFFRBJYgoARhCYoNr6HkoGHnFmyaJwXn+y9JDI7H46fD6fRP9hTrhyb6w0YF+1Gq1U1ACULd/ltV+/PhHHaww7jzHYTQpeLdEljWcE8MDklSwC6eGLx/8+Y7H96+/UvaJCIgAusRUIKwHtuqV06Tg9PhYK+qTZLyhRIgKbD77aPJKU0MPCkgOVViUKgDpVazBJQgNOva6w07H9Rh+smSA/06YwDSUHFPU949Pv6L3WufSQpMj98zubw8MVBScEGigghsTkAJwubIy97QDmzLB7o6Kjno8lDtNgKeGNiN9ie20uVjK08K9LTAqOglAgUQUIJQgBNKUSGXHHBYl6Kf9EgJ1FW3++uXJp/TxMCs+MyXDvW0wEjoJQIFEVCCUJAz9lTFDm47t7sabJ0c8JcaU0GvPvGxXa1VK4mAPy3Ah6bX900uTwysfLLKv9p99qW+dGg09BKBwggoQSjMIXuo83x4d7a2Q9vO7k7T1RUP5OwzJLbhMZWhTX3s0JrsPbTGnn0t7+2JgWWdnY8RzGZrOvyK+8vki/cPD39qbXqJgAgUSEAJQoFO2VKlXAC1g9ti73wtWAtJA7Ytdg7881e8fQZ7p/rcvqpW6CMwlBiYL3ha8IXdXz/om692ERCBcggoQSjHF5trQjC3Q9teL1vb4d2pv/S8LjE/Bl+buEgiYD9inlJBryje/1qr8RbXeXzk0Aj1RQLGtO/7Bf4xgp4WRGAqi0AFBJQgVOCkNVQkuBPQ49oE4FhPy8yxQHBySeen473uwZz1pwi/NZGKr+VX7x9aj319fO7qdmBXrl9twwT8aQEcbWTf9wuUGBgcvUSgRgJKEGr02o06ExDT4E6gTZdlHIe/SzonHU+doMxaUTyY07+lsG/Ug7LvH6/Y5TbGdpXzBDwxMF/r+wV5RGoVgSYIKEFowo3TjSDoExDjDA+c9Hmg5JqOi3MoW4A4fxTAfBeCMn2liuvZpx92I33999w+lBjYvaLvF9zzzSHbmySgBKFJt/YbZQe5vbr9BETEOuzV7Yu1NCEgGUDimG3Kt++iRGE6Q7s39P2C6bg0UgSaIaAEoRlXjhtiB73F+PFxPsIGd54QkAwg3t/C1RMFrjl7eKqSa2+9zZ8WPN8z+n5B6w6XfSKQIaAEIQOllSaCG8Ihj4zZtVVCMKbHXv0kCUjc3x6pHGEY21oue2Jg94K+X9Cyo2WbCEwgoARhAqSahhDMEBICghvSp78FgeafEPTZPtSeSxKGxrfQ9+7jx3/nnrF74lViYPeQvl/QgpNlgwjMJKAEYSawEoeTECAc8HaYD/4tAgsAJwIgwscFyDyb7mM0fKKlsI31Vspm1/+ZnOy/P0xs0t8vSICoKgL3RkAJQqUe94SAw30sKYgmKiGINIbLrSYJ/rSAe8cI/JbJy+t4VGLwQkMlEbhrAkoQKnJ/mhT0qe5PCdJ+Al7apvowgZTZc1AdnlRorycGmacFh+Px+B/Y+uHNG/1ho0L9J7VEYGsCShC2Jj5zv7lJAYc8TwnSQEb7zK01/JkACddz8XzBJ+dCJf9MSQzev3nzR5WYIzVFQAQ2IqAEYSPQc7YhABHgET4+eJnbLRG4CPwISYH3Ms/LXOnnKrmOQGTLCkM+ob8E8aSAe2HoiYESgxK8JR1EoEwCShAK8cutSYGbwTpe5koSwVVyG4FakixPDHJJgRH4tX+UoMTAaOglAiIwSEAJwiCeZTvT1Qjm/ISHDP1USpAnQCHpT7Ppmuk6Y+PT+arXSWAoMfCkwO6f7ykxqNO/0loE9iCgBGFj6mskBW4CiYaXuVpAsHyBkmQLAvjWBV9sKbknBp4YKCnYwvvaQwTaI6AEYbJPrx9I0PBgYRHbXvm15jwpSFdg/dim5CDSuK2M/5C4CrxTMcceXeLYvcokDa7jXjpoXxEQgXoJKEFYyXcEFD+cCRq5bUgIEII5cu3HAewT12etWFe5nwB+coFjTvAf0r9K+T3RLuwtX2NpKAIisDeBu0kQtgDNwesHcV9AISFACOIkBMgturFnnM/asX6vZbi4uE9yV/zksgQr+Lvg4yXE9PtFn25H//sFDw9H36tvrLfbesfIwtt1FQEREIFIQAlCpHFFmSDkhy0Hb26JGDBICJDcuGva0j2XXPsafbaYA3MXZ59e4eKyhE74MK5D3QNyvMLfJY6/tmx2fbK9fpTO98Qg9/2CqA/ldG5atz1OLnBN+1UXARG4TwKVJAhlOYdD1A9UglBOOzvUL/8jpCUDRtwLHWJ9SjCI40stwxfBvpzA3GUJG9xXXGGYE3xI/xL7TVnD7P5kYlsevozjze5foF8uMWAc3FKxRexF77jY+p2nC+hQkkTbxq3RCBEQgVsIKEGYQY/DicOSQzQ3zU7h1ZMC3xc9vMyVoMG1dIGhCzbkBL7Irba4P7jCp08I/i5T91xCP/ZyFvEKE+vrJAZWP7/Mlh/R3yfolZPz5Ab+ibb1MUjbI9sGEMgEEdiMwCYJwmbWrLQRBwyHDodTuoUd2JslBb43+niZK4GPawmCbgi8cgJDl1v0jdyxPyce9LneslffXOxEcnZObXMW8dq3n9qvIxDZpn7Bf9etqlki0D4BJQgDPubw4EDhgEmHEaAISgQfJO1fs57TZ839fG14uMAlJ+iG+Jxbr3B2iWuxB5LTYa029svpENtKKTuzsSv3cJ/MtaVvnSXaox1z9Roaj0/j/TI0Vn0icG8EJiQI94bkcCAIcmhweKTWc1Bx4G2dFLge6OVlrujC9VbBZhf2yAk8XG7db+p834/r1Dm1j+MeQ/DttcL9OUWGWKV7D42lz+8ZyktLtCXVq68OQ5ep+rgNXKfO0TgRaJWAEoTgWQIkB0MuGHHQcBBxUIUpmxbRLW6IPl5H9yiMnSPY7OJr6jpMgHsiCv6YIsY5+2uLtDOfewwZ3n37XnRzwe4+Dbjv+vq2bIehi+sdr0M2oCd28J6iLBGBJgmMGKUEwQBxCHAY2AFtL2sILw4RDhUOmtC8eBEdoqBPKummsd8UP0ZJx9ZQh/UcwS9bS+TIPREl9vWV8ZnZmP7a4m+w4/3Dwx/0zSutHbvR2SXVDzu5n9P2kupjNpSkq3QRgT0I3HWCwAHGQUZgTeHbIX7i8OMQSfum1FnbhT3GBB2iTNljizFw6BP4LCmwniNb2L/UHuZ//7XFzpLmc35t8atOY4UVvw+i6mbb+VcmY1vJZbeB+71kPaWbCDwTWP1ylwkCgdsO7BMHWEqYw4GDgkCV9nmd+S6skxPWdvF5e1yxxwW75goc+mQPe2rb893j439yf5jenV9btHuDxOBY01MDs2H0xf2VDuK9krapLgIiUD6Bu0oQOKg4rO1wtlfXOR5EafVxjM2JTb48zmf81uK6cuVAHpIY3LfWs7X9uC+m2uSJgfmo83GC3TtNJgaRC/djrKssAiKQIVBB010kCBzsBHo7nO2V94p1XII+5fyo9VotkJz/ngJXDlgk3Y02REE/JbNNPd4X+KlvV7vXcn8eubrvGfTZN6Wd+9THRW7eVvK1Nn1LZind6ibQdIIwJTFY030EERcOzCFJgz66R91YJ9ZV3pcA/ko18KcG1p77OKH67xmYXc2/LLmzt9qLmTk/v/SqdMcE7sL0JhMEgitv9CV/ErBT4/ITPuWhYO99HC4uc++mVHfWmbuGxi9HgPupbzVPDOy+uLuPE/qY1NjOuVGj3tJZBNYi0FyCwEGeBlfg2eF9/q0ED95zrwToKKy5lmBDXBtdY13lfQlEf5ivPtu91UkMTLu7+jjB7B19lR58zY+vvrQc/TxqoAbURUDaTiLQVILAmzy12g7vc2JAcE/7SqynNuiQ2t9LqU8SjSwffWmxCl9C1McJhoT3nl2KfpG45Pyr913RbpNyGxFoIkHIvck5nHiT15IY5PyN/rl2te1HIPrEAsvnoMk5EW3t1xaDfTcVLXGy101LLDrZzwxTyl7dpaOPuz2qFUJAamxEoPoEwQ7p7KPBGhMDbNnI79pmIoE+n1g7ycEluFhQqf69NBHJ5GGlvgfNd6/ODIwyHx4RyhIREIHDoepDjTd66sRW3uCtVM30UQAADZxJREFU2JH6p+Z64pPjxZbj8ZtLWYULgdz789K5QwF9kHRrf9qYtqu+EgEtWw2BahOE3Bs9OcCrcQKK5uyhvUTh8ewUKVH3OTr1+cTaeXrgS50+vHnz+17RNU9gz/cm96r5zPKArm7WcEKvUp90dLVVTQS2J1BdgpB7s/sbfXt86+zIobXOyuOrOl8O1D6xH507f1Sqr943P21nz5yMa7vdCPeJ6U5yYCY/7W3t1b2HnjRf91/jZG/LdfcYW517Cj3MWfbqjja/HZUYdJlMrGnYHRGo6nDLvdlbeKNj19b3HIcnwt5R7CS117ba2IbZhCPqtWQZu/vELWc/LydXU/e5RR8tPIMYvvAeHR6xfC/+M0fZq7s2uiDdVtVEQARyBKpJEHjDpwa0+Eafa1Mu0MFqTOzkPAfllOk91N323NW5pRzgbH08PfCukz5acBTdq3Ha7ekBeyNdjQ4HU+g0972VrtFEXUaIwAwCVSQIuTd8C2/256BjZ9eLx7B1juSC3MtqKi1FAM62ll3s36fXET/hw6eq/s0R2Op9ih/wR6qDvbnOiYE+TkjJqC4C4wSKTxDSN72/4cdNW2cEB1FO0HOuWLSx1zp6LrUqvPuEw38tuUV/9E31oq1PbtnLHHhOFNz3t6zVwlw4bGkH70X2xA9xX3zNPdBYYhBNVFkEVidQfIKQEuAg4EBw4YDoEx+z5JX9c5LquWWdw9BlaF/GcGjOEQ7YPhna69a+nI7oP2Vd/JP6nHl9dqR7MdaFvqn7MifuS/2eBXZr2g9rfJ3uwb74Om1XXQREYB6B6hKE1DwOiD5Jx5ZcJwi5cMDNET8M4ZCzkXVZz8flxtTQhv7YEWWq3rAhoLj0zaM/7WPf2Ob7wzW2p2XWckn7Wqxj6xZ2sQ+S7oU/8E3aXkxdiohAZQSqTxD24s1hlAqH01RJ9SYIuaR9Y3UOSwJgHIdurgvrxr6Wym6jX7F7in0wc+EJVG4Oa+bavQ2ujHHx9tzV9+Ka62+tDSZL2oSPYIek6+Jz9sMfaZ/qIiAC1xMoPkHgjd8nHAxzpW+tue0cRqlc6wb2vnZu7sBkPXS7ds2a52E39kfhHhmyieQKjsjQuLG+uOfQWPZBCHpD42rqw56l9YUP6yL4KF0fv8Icn6d9K9S1pAjcHYHiE4Qhj3AwzJWh9bbq48BbYq90HT8wl1i7pTW4RwgkLlNtgy8ydXwc53txje2xTNBjfYRgGPtqLg/ZPGYXHBCYwCc33u9z/JrrV5sIiMAyBKpOEJZBsO8qtxymUXPW0YEZifSXYeVCsOkf+dRDsHoqPf1LAHsqTfvX9+LaN4NgyD5I35hS25fQGaasAwcktRU/ITC86j5PF1RdBERglIAShFFEZQ7gMC1Ts7q0ItgQdOZoTQCDfyoEubF12Mulb+yUdfrmbt0Og7gntsX6UBk7mY/ANDc2JgX4KjdGbSIgAusQUIKwDtfeVTkMezuv7JhzKF+5xV1Ng6cLAWqq8QQ5/DtV+tatJRBiZ7QBZrGeK89JCljvmUVuKbWJgAisTEAJwsqAh5bnABzqV9/+BAhQZz8dj/+1hTbnvbbY6MY95iYHnhiQROW2JhHDdgTmuTFqEwER2JaAEoQNeaeH6oZba6sbCXx48+Z30yUIZi4EuLR/Sp15iK8zZc7eY9L7GN1zOnlS8PXj42ksMVBSkCOoNhHYl4AShJ349x2q16jDQXzNPM2ZRyD1WQyUBDj65wrzkHma7DPa7P1kYvnMy/7Y+1I7HLgXGYOMJQXMrcX2aKPKInAvBJQgVOppO6Xt9aR830H81Kt/lyRgrP8nrkcgjPUGy2eTzM5PVvjS5PIiwMeEwMaMPilgjpKCC0IVRKBoAkoQNnIPh+eSW6WH7NLrL6lrDWtZtmWvJ02HWL5/ePj+vSUJxuNVcgApa+9NCOg3oOf/k6KSAmhIRKA+AkoQdvAZB+YS26brcGAvsa7WeHpU3seBJCHH/t3j46/65uzWfuPGPCGwJTpPDqze+yIpQOCTJrG9k9QhAiJQJAElCEW6ZbpSHMZxtJKESGN6mWAWWdpTguNzcOxdhCAYO23+79TOH5sR7EDgEG1My2bzCYEFAkckHae6CIhAfQSUIGzgMw7ctbbhMOaAjutzsMe6ytMIwDKOHAuOjCUoco0CfyS2XVlefRr3JoK+CDYjfRtzryHYjcAM6RuvdhEQgXoJKEHYwHfxwOVwXXpLDuh0XQ77pfe5h/UIetHOKRzTOT6fuS7etveVZABxvbg3kTG9sBHhXkPGxqtfBESgfgJKEDb24VqHK+tygEdzPAjENpXHCfRxhGffbOYgnf5QYa5LaF69SDKA+N4kA8iMjX8zZNeMdTRUBESgMgJKECpz2Ji6ucOc4DA2T/1dAukTGe+FJeL19Ap/JG2Pdea7xPZbyyQCiK/NlWQAmbv28XT6hB0mX82dq/EiIAJtEFCC0IYfO1bYoW4xodN0IFgQPLqtqvUR+OnDwxc5jj4enlFStsx18Tm5a1jjf3P93sb6LmHOKZbN6UfE51xz9cTg/du337lmvuaIgAi0Q0AJQju+7FhCcEp/CiZ4EFA6A1UZJABHl6GBzha+qeAHhHUG1vjtdF6ss77LwBpXdykxuBqdJopAswSUIKzsWn7qW3mL3uVz30tgsAceys3KCoYR4JG5S3tgh/vcuWuPV2KwNmGtLwL1ElCCsKHv+Clyw+0uW/UFtRID1kXpggvwjLKXX69GdDp9ezDBBn2UcDVFTRSB5gkoQWjexU8GEgyQp9rLvyQJyEtLEaWqlPAnNfBNheQBmWIQ45ApYwfHWPD3BCDV51x/+/a7H0wG11CnCIjA3RNQgrDyLUDw8C141Ozlva7nAPHwYKp0NSBJQLqtqt1KAP8jzn3oyjjEx1iQ//VZUiWeEwDr+9bHdq4W/JUApNBUFwERmEtACcJcYo2MJ6DkTCFJQHJ9k9s0cBECFuS/d5aHhyP+ushzAmB9311kIy0iAiIgAhkCShAyUO6lyQNOzl6SBCTXpzYREAEREIH2CShB2NjHe/5WQ5+pSaLQGUaSgHQaVREBERABEWiegBKEDVy8yBfPNtBTicIGkLWFCIiACFRCQAnCxo46Hg72Oqz33wIrT0kU9FRhAdBaQgREQAQKJqAEYQPn8M30uE2JHzNE/bw8lCgwhiShFlvQVyICIiACIjCdgBKE6awWG2mPEOyVXa7IxqFEwQw5kigUqbiUEgEREAERuJqAEoSr0c2bSJCNM2oMqtiA5L5TgT0u0U6VRUAEREAE6iSgBGFJv42sRXCNQ2p9PM9HJqkt0S4lCpGGyiIgAiJQJwElCBv7Lf70zeP5jbdfdDuSBKRvURKFWpOgPpvULgIiIAL3QkAJwounNynx03fciCAa6zWWSRJcUv1JglqwMbVLdREQARFonYAShB08TDCN2xJAkdhWaxnbkFT/VuxL7VJdBERABFol0E6CUJmHWg+irdtX2e0mdUVABERgNgElCLORLTehL4i28tM29iGRWCu2RZtUFgEREIEWCZSSILTIdpJNaQD1SQTSVr7gl9qIbW6nriIgAiIgAmUSUIJQgF8IoEiqSktf8EvtU5KQelt1ERABESiLwDIJQlk2VasNQRRJDSCYIrU/UUhtw6bUVtVFQAREQATKIKAEoQw/dLRIA6l3+hMFAivi7TVd49+BqElv6SoCIiAC90aABOHebK7CXpIEZEhZkgSXoXEl9aV/B6L2pyIlsZUuIiACIrAkASUIS9JcYS2SBGTsJ29PFPxaYuBFJ/SLmHgqEusqi4AIiIAILEXgtnWUINzGb7PZ/ORNouAytjGBl2CcCkF6bO6S/eznOqDTkmtrLREQAREQgfUIKEFYj+2qK3uiwHXORgRpD9h9V4J6TnyfXF/fWuzn8+KVJyLojsR2lUVABERABJ4I7P2vEoS9PbDA/gRZFwIvcsuyBPWceBKQ65uyH3q5njwRmTJHY0RABERABPYhoARhH+6r7UrgRTwQxysBerWNexZmTwQ90KtnmJpFQAREoDEC9ZujBKF+H062gABNoB4SgnmUocXjOMq5ddkTGVpHfSIgAiIgAuURUIJQnk921YhgHiUX9L0tjqO8q+LaXAREQAQWJKClDgclCLoLREAEREAEREAEXhFQgvAKiRpEQAREQATqJiDtlyCgBGEJilpDBERABERABBojoAShMYfKHBEQARGonYD0L4OAEoQy/CAtREAEREAERKAoAkoQinKHlBEBERCB2glI/1YIKEFoxZOyQwREQAREQAQWJKAEYUGYWkoEREAEaicg/UXACShBcBK6ioAIiIAIiIAIXAgoQbigUEEEREAEaicg/UVgOQJKEJZjqZVEQAREQAREoBkCShCacaUMEQERqJ2A9BeBkggoQSjJG9JFBERABERABAohoAShEEdIDREQgdoJSH8RaIuAEoS2/ClrREAEREAERGARAkoQFsGoRURABGonIP1FQAS6BJQgdHmoJgIiIAIiIAIiYASUIBgEvURABGonIP1FQASWJqAEYWmiWk8EREAEREAEGiCgBKEBJ8oEEaidgPQXAREoj4AShPJ8Io1EQAREQAREYHcCShB2d4EUEIHaCUh/ERCBFgkoQWjRq7JJBERABERABG4k8P8AAAD//w6ADNMAAAAGSURBVAMAmK/BYxrobpUAAAAASUVORK5CYII=</t>
+        </is>
+      </c>
       <c r="AS16" t="inlineStr"/>
       <c r="AT16" t="inlineStr"/>
       <c r="AU16" t="inlineStr"/>
@@ -2543,7 +2747,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>A DEFINIR</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H17" t="inlineStr"/>
@@ -2682,7 +2886,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>ARQUIMEDES</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -3214,7 +3418,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>EQUIPE EMED PLANTÃO</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -3564,12 +3768,12 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>EQUIPE EMED PLANTÃO</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>(85) 3254-2929</t>
+          <t>85999150273</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -3696,11 +3900,7 @@
       <c r="AR24" t="inlineStr"/>
       <c r="AS24" t="inlineStr"/>
       <c r="AT24" t="inlineStr"/>
-      <c r="AU24" t="inlineStr">
-        <is>
-          <t>NENHUM (INDIVIDUAL)</t>
-        </is>
-      </c>
+      <c r="AU24" t="inlineStr"/>
       <c r="AV24" t="inlineStr"/>
       <c r="AW24" t="inlineStr"/>
       <c r="AX24" t="inlineStr"/>
@@ -3739,12 +3939,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>EQUIPE EMED PLANTÃO</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>(85) 3254-2929</t>
+          <t>85999150273</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -3871,11 +4071,7 @@
       <c r="AR25" t="inlineStr"/>
       <c r="AS25" t="inlineStr"/>
       <c r="AT25" t="inlineStr"/>
-      <c r="AU25" t="inlineStr">
-        <is>
-          <t>NENHUM (INDIVIDUAL)</t>
-        </is>
-      </c>
+      <c r="AU25" t="inlineStr"/>
       <c r="AV25" t="inlineStr"/>
       <c r="AW25" t="inlineStr"/>
       <c r="AX25" t="inlineStr"/>
@@ -4479,12 +4675,12 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>EQUIPE EMED PLANTÃO</t>
+          <t>NETTO</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>(85) 3254-2929</t>
+          <t>85999150273</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -4607,11 +4803,7 @@
       <c r="AR29" t="inlineStr"/>
       <c r="AS29" t="inlineStr"/>
       <c r="AT29" t="inlineStr"/>
-      <c r="AU29" t="inlineStr">
-        <is>
-          <t>NENHUM (INDIVIDUAL)</t>
-        </is>
-      </c>
+      <c r="AU29" t="inlineStr"/>
       <c r="AV29" t="inlineStr"/>
       <c r="AW29" t="inlineStr"/>
       <c r="AX29" t="inlineStr"/>
@@ -4619,6 +4811,908 @@
       <c r="AZ29" t="inlineStr"/>
       <c r="BA29" t="inlineStr"/>
     </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>66</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CDI PETROLINA</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>MAMÓGRAFO - VMI COMPACTO  [N/S: 123456414 | FAB: 2008 | LOCAL: SALA 03 | STATUS: EM FUNCIONAMENTO]</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>(85) 3254-2929</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>UNIDADE HOSPITALAR</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>KEZIO</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>9896659858</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>[PORTAL CLIENTE] NAO ESTA COMPRIMINDO</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>🟢 Não foi observada  | 🟢 Movimentação mecân | 🟢 Comandos e botões</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr"/>
+      <c r="U30" t="inlineStr"/>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>[PORTAL DO CLIENTE] nao esta comprimindo | Solicitante: kezio</t>
+        </is>
+      </c>
+      <c r="W30" t="inlineStr"/>
+      <c r="X30" t="inlineStr"/>
+      <c r="Y30" t="inlineStr"/>
+      <c r="Z30" t="inlineStr"/>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>9896659858</t>
+        </is>
+      </c>
+      <c r="AB30" t="inlineStr"/>
+      <c r="AC30" t="inlineStr">
+        <is>
+          <t>CONTRATO MANUTENÇÃO</t>
+        </is>
+      </c>
+      <c r="AD30" t="inlineStr">
+        <is>
+          <t>MALETA PADRÃO EMED</t>
+        </is>
+      </c>
+      <c r="AE30" t="inlineStr"/>
+      <c r="AF30" t="inlineStr"/>
+      <c r="AG30" t="inlineStr"/>
+      <c r="AH30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI30" t="inlineStr">
+        <is>
+          <t>NAO ESTA COMPRIMINDO</t>
+        </is>
+      </c>
+      <c r="AJ30" t="inlineStr">
+        <is>
+          <t>OPERANDO COM FALHA</t>
+        </is>
+      </c>
+      <c r="AK30" t="inlineStr"/>
+      <c r="AL30" t="inlineStr"/>
+      <c r="AM30" t="inlineStr"/>
+      <c r="AN30" t="inlineStr"/>
+      <c r="AO30" t="inlineStr">
+        <is>
+          <t>Aberto pelo Portal do Cliente em 22/10/2026 01:39.</t>
+        </is>
+      </c>
+      <c r="AP30" t="inlineStr">
+        <is>
+          <t>EM ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AQ30" t="inlineStr"/>
+      <c r="AR30" t="inlineStr"/>
+      <c r="AS30" t="inlineStr"/>
+      <c r="AT30" t="inlineStr"/>
+      <c r="AU30" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV30" t="inlineStr"/>
+      <c r="AW30" t="inlineStr"/>
+      <c r="AX30" t="inlineStr"/>
+      <c r="AY30" t="inlineStr"/>
+      <c r="AZ30" t="inlineStr"/>
+      <c r="BA30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>71</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HOSPITAL UNICLINIC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>RX FIXO ALTUS</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>PREVENTIVA COM REPARO</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>LEONARDO</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>(85) 3254-2929</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>FORTALEZA - CE</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>RICARDO</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>8678198733</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>[P3 - PREVENTIVA PROGRAMADA] BOTÃO DE ACIONAMENTO DO FREIO HORIZONTAL</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Movimento : ⚪ Não / Nenhuma das opçõe | Sentido do: ⚪ Não / Nenhuma das opçõe | Intermitên: ⚪ Não / Nenhuma das opçõe</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr"/>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>LEONARDO - CFT</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>[EMEDONLINE - RAIO-X] Botão de acionamento do freio horizontal | [Movimento Manual da Mesa: ⚪ Não / Nenhuma das opções] [Sentido do Avanço: ⚪ Não / Nenhuma das opções] [Intermitência do Defeito: ⚪ Não / Nenhuma das opções] | Solicitante: Ricardo</t>
+        </is>
+      </c>
+      <c r="W31" t="inlineStr"/>
+      <c r="X31" t="inlineStr">
+        <is>
+          <t>Não cadastrado</t>
+        </is>
+      </c>
+      <c r="Y31" t="inlineStr"/>
+      <c r="Z31" t="inlineStr"/>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>8678198733</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr">
+        <is>
+          <t>Fortaleza - CE</t>
+        </is>
+      </c>
+      <c r="AC31" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD31" t="inlineStr">
+        <is>
+          <t>SUGESTÃO: MANUTENÇÃO DE ELETROFREIOS &amp; MECÂNICA (ESTATIVA / MESA)</t>
+        </is>
+      </c>
+      <c r="AE31" t="inlineStr">
+        <is>
+          <t>PREVENTIVA / CALIBRAÇÃO (RAIO-X)</t>
+        </is>
+      </c>
+      <c r="AF31" t="inlineStr"/>
+      <c r="AG31" t="inlineStr"/>
+      <c r="AH31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI31" t="inlineStr">
+        <is>
+          <t>BOTÃO DE ACIONAMENTO DO FREIO HORIZONTAL</t>
+        </is>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>OPERACIONAL COM PENDÊNCIA (AGUARDA PREVENTIVA)</t>
+        </is>
+      </c>
+      <c r="AK31" t="inlineStr"/>
+      <c r="AL31" t="inlineStr"/>
+      <c r="AM31" t="inlineStr"/>
+      <c r="AN31" t="inlineStr"/>
+      <c r="AO31" t="inlineStr">
+        <is>
+          <t>Chamado aberto via EmedOnline (RAIO-X) em 22/10/2026 01:53.</t>
+        </is>
+      </c>
+      <c r="AP31" t="inlineStr">
+        <is>
+          <t>EM ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AQ31" t="inlineStr"/>
+      <c r="AR31" t="inlineStr"/>
+      <c r="AS31" t="inlineStr"/>
+      <c r="AT31" t="inlineStr"/>
+      <c r="AU31" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV31" t="inlineStr"/>
+      <c r="AW31" t="inlineStr"/>
+      <c r="AX31" t="inlineStr"/>
+      <c r="AY31" t="inlineStr"/>
+      <c r="AZ31" t="inlineStr"/>
+      <c r="BA31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>72</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>JOÃO DA LUZ</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>TAUA</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>TC CT/E</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>(85) 3254-2929</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>FORTALEZA - CE</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>KATIA</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>85987654689</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>[P1 - EMERGÊNCIA MÉDICA] SOFTWARE NÃO FINALIZA O STARTUP.</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Inicializa: 🔄 Computador liga, mas o  | Código de : ⚪ Não / Nenhuma das opçõe | Intermitên: 🔴 Permanente (não abre ne</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>EQUIPE EMED PLANTÃO - CFT</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>[EMEDONLINE - TOMOGRAFIA] Software não finaliza o startup. | [Inicialização do Sistema: 🔄 Computador liga, mas o software de aquisição médica não abre ou congela no boot] [Código de Erro no Painel: ⚪ Não / Nenhuma das opções] [Intermitência do Defeito: 🔴 Permanente (não abre nem após reiniciar o PC)] | Solicitante: Katia</t>
+        </is>
+      </c>
+      <c r="W32" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\FOTO_EMEDONLINE_20261022_070913_IMG_20261019_022653_242.jpg</t>
+        </is>
+      </c>
+      <c r="X32" t="inlineStr">
+        <is>
+          <t>Não cadastrado</t>
+        </is>
+      </c>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>85987654689</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>Fortaleza - CE</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD32" t="inlineStr">
+        <is>
+          <t>SUGESTÃO GERAL DE ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AE32" t="inlineStr">
+        <is>
+          <t>CORRETIVA EMEDONLINE (TOMOGRAFIA)</t>
+        </is>
+      </c>
+      <c r="AF32" t="inlineStr"/>
+      <c r="AG32" t="inlineStr"/>
+      <c r="AH32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI32" t="inlineStr">
+        <is>
+          <t>SOFTWARE NÃO FINALIZA O STARTUP.</t>
+        </is>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>PARADO (INOPERANTE)</t>
+        </is>
+      </c>
+      <c r="AK32" t="inlineStr"/>
+      <c r="AL32" t="inlineStr"/>
+      <c r="AM32" t="inlineStr"/>
+      <c r="AN32" t="inlineStr"/>
+      <c r="AO32" t="inlineStr">
+        <is>
+          <t>Chamado aberto via EmedOnline (TOMOGRAFIA) em 22/10/2026 07:09.</t>
+        </is>
+      </c>
+      <c r="AP32" t="inlineStr">
+        <is>
+          <t>EM ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AQ32" t="inlineStr"/>
+      <c r="AR32" t="inlineStr"/>
+      <c r="AS32" t="inlineStr"/>
+      <c r="AT32" t="inlineStr"/>
+      <c r="AU32" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV32" t="inlineStr"/>
+      <c r="AW32" t="inlineStr"/>
+      <c r="AX32" t="inlineStr"/>
+      <c r="AY32" t="inlineStr"/>
+      <c r="AZ32" t="inlineStr"/>
+      <c r="BA32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>73</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>JOÃO DA LUZ</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>TAUA</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>TC CT/E</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>PREVENTIVA (Com Checklist POP/IT)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>ARQUIMEDES</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>5585977777777</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-11-21</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>SEDE EMED</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>[CICLO PREVENTIVO AUTOMÁTICO] PROGRAMADO PARA ETAPA 1: MESA DE EXAMES, COMANDOS E CONSOLE</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr"/>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD33" t="inlineStr"/>
+      <c r="AE33" t="inlineStr">
+        <is>
+          <t>ETAPA 1: MESA DE EXAMES, COMANDOS E CONSOLE</t>
+        </is>
+      </c>
+      <c r="AF33" t="inlineStr"/>
+      <c r="AG33" t="inlineStr"/>
+      <c r="AH33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI33" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO PREVENTIVA PROGRAMADA — ETAPA 1: MESA DE EXAMES, COMANDOS E CONSOLE</t>
+        </is>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>OPERACIONAL</t>
+        </is>
+      </c>
+      <c r="AK33" t="inlineStr"/>
+      <c r="AL33" t="inlineStr"/>
+      <c r="AM33" t="inlineStr"/>
+      <c r="AN33" t="inlineStr"/>
+      <c r="AO33" t="inlineStr"/>
+      <c r="AP33" t="inlineStr">
+        <is>
+          <t>LIBERADO PARA USO NORMAL</t>
+        </is>
+      </c>
+      <c r="AQ33" t="inlineStr"/>
+      <c r="AR33" t="inlineStr"/>
+      <c r="AS33" t="inlineStr"/>
+      <c r="AT33" t="inlineStr"/>
+      <c r="AU33" t="inlineStr"/>
+      <c r="AV33" t="inlineStr"/>
+      <c r="AW33" t="inlineStr"/>
+      <c r="AX33" t="inlineStr"/>
+      <c r="AY33" t="inlineStr"/>
+      <c r="AZ33" t="inlineStr"/>
+      <c r="BA33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>77</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>HOSPITAL SAO CARLOS</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>COMPACTO PLUS 300</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>PREVENTIVA (Com Checklist POP/IT)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>ANTONIO</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>85996199711</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>NÃO</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-11-21</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>AVENIDA PONTES VIEIRA, 2531 - DIONISIO TORRES, FOTALEZA</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>SRA. DAMARES</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>[CICLO PREVENTIVO AUTOMÁTICO] PROGRAMADO PARA ETAPA 1: MESA DE EXAMES, COMANDOS E CONSOLE</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr"/>
+      <c r="U34" t="inlineStr"/>
+      <c r="V34" t="inlineStr"/>
+      <c r="W34" t="inlineStr"/>
+      <c r="X34" t="inlineStr"/>
+      <c r="Y34" t="inlineStr"/>
+      <c r="Z34" t="inlineStr"/>
+      <c r="AA34" t="inlineStr"/>
+      <c r="AB34" t="inlineStr"/>
+      <c r="AC34" t="inlineStr">
+        <is>
+          <t>CONTRATO</t>
+        </is>
+      </c>
+      <c r="AD34" t="inlineStr"/>
+      <c r="AE34" t="inlineStr">
+        <is>
+          <t>ETAPA 1: MESA DE EXAMES, COMANDOS E CONSOLE</t>
+        </is>
+      </c>
+      <c r="AF34" t="inlineStr"/>
+      <c r="AG34" t="inlineStr"/>
+      <c r="AH34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI34" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO PREVENTIVA PROGRAMADA — ETAPA 1: MESA DE EXAMES, COMANDOS E CONSOLE</t>
+        </is>
+      </c>
+      <c r="AJ34" t="inlineStr">
+        <is>
+          <t>OPERACIONAL</t>
+        </is>
+      </c>
+      <c r="AK34" t="inlineStr"/>
+      <c r="AL34" t="inlineStr"/>
+      <c r="AM34" t="inlineStr"/>
+      <c r="AN34" t="inlineStr"/>
+      <c r="AO34" t="inlineStr"/>
+      <c r="AP34" t="inlineStr">
+        <is>
+          <t>LIBERADO PARA USO NORMAL</t>
+        </is>
+      </c>
+      <c r="AQ34" t="inlineStr"/>
+      <c r="AR34" t="inlineStr"/>
+      <c r="AS34" t="inlineStr"/>
+      <c r="AT34" t="inlineStr"/>
+      <c r="AU34" t="inlineStr"/>
+      <c r="AV34" t="inlineStr"/>
+      <c r="AW34" t="inlineStr"/>
+      <c r="AX34" t="inlineStr"/>
+      <c r="AY34" t="inlineStr"/>
+      <c r="AZ34" t="inlineStr"/>
+      <c r="BA34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>78</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CLINICA IMEDIATA</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>TOMOGRAFO - GE - BRIGHTSPEED</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>ANTONIO</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>UNIDADE HOSPITALAR</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>PEDRO</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>8898654682</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>[CHAMADO ABERTO] MESA TRAVANDO O MOVIMENTO DE UP E DOWN</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+      <c r="T35" t="inlineStr"/>
+      <c r="U35" t="inlineStr"/>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>⚠️ Sim, e também não responde pelo painel do Gantry (travamento total) | ⬇️ Acontece na descida (DOWN) | ⚖️ Acontece apenas com paciente / peso sobre a mesa</t>
+        </is>
+      </c>
+      <c r="W35" t="inlineStr"/>
+      <c r="X35" t="inlineStr"/>
+      <c r="Y35" t="inlineStr"/>
+      <c r="Z35" t="inlineStr"/>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>8898654682</t>
+        </is>
+      </c>
+      <c r="AB35" t="inlineStr"/>
+      <c r="AC35" t="inlineStr"/>
+      <c r="AD35" t="inlineStr">
+        <is>
+          <t>SUGESTÃO GERAL DE ATENDIMENTO</t>
+        </is>
+      </c>
+      <c r="AE35" t="inlineStr"/>
+      <c r="AF35" t="inlineStr"/>
+      <c r="AG35" t="inlineStr"/>
+      <c r="AH35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI35" t="inlineStr">
+        <is>
+          <t>MESA TRAVANDO O MOVIMENTO DE UP E DOWN</t>
+        </is>
+      </c>
+      <c r="AJ35" t="inlineStr">
+        <is>
+          <t>OPERANDO COM FALHA</t>
+        </is>
+      </c>
+      <c r="AK35" t="inlineStr"/>
+      <c r="AL35" t="inlineStr"/>
+      <c r="AM35" t="inlineStr"/>
+      <c r="AN35" t="inlineStr"/>
+      <c r="AO35" t="inlineStr"/>
+      <c r="AP35" t="inlineStr">
+        <is>
+          <t>LIBERADO PARA USO NORMAL</t>
+        </is>
+      </c>
+      <c r="AQ35" t="inlineStr"/>
+      <c r="AR35" t="inlineStr"/>
+      <c r="AS35" t="inlineStr"/>
+      <c r="AT35" t="inlineStr"/>
+      <c r="AU35" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV35" t="inlineStr"/>
+      <c r="AW35" t="inlineStr"/>
+      <c r="AX35" t="inlineStr"/>
+      <c r="AY35" t="inlineStr"/>
+      <c r="AZ35" t="inlineStr"/>
+      <c r="BA35" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(v23): rota inteligente via WhatsApp, geofencing calibrado em 250m e botao de encerramento rapido para equipamento em uso
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -749,18 +749,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>[CONCLUÍDO COM PENDÊNCIA: PROGRAMADA] BOTAO ANTIVANDALIMO 22MM | REALIZADO SUBSTITUIÇÃO DO BOTÃO DO HANDSWITCH (PERA).
-- REALIZADO SUBSTITUIÇÃO DA GRAXA ISOLANTE DOS CONECTORES DO CABO FEDERAL DO ANODO E CATODO.
-- REALIZADO TESTES OPERACIONAIS DE FUNCIONAMENTO.
-- REALIZADO ACOMPANHAMENTO DE EXAMES COM PACIENTES OK | [DIAGNÓSTICO: REALIZADO SUBSTITUIÇÃO DO BOTÃO DO HANDSWITCH (PERA).
-- REALIZADO SUBSTITUIÇÃO DA GRAXA ISOLANTE DOS CONECTORES DO CABO FEDERAL DO ANODO E CATODO.
-- REALIZADO TESTES OPERACIONAIS DE FUNCIONAMENTO.
-- REALIZADO ACOMPANHAMENTO DE EXAMES COM PACIENTES OK] | [FATURAMENTO BOLETO BANCÁRIO (VALOR INTEGRAL) — VALOR FINAL: R$ 0.00]</t>
+          <t>[REAGENDAMENTO NECESSÁRIO] Visita presencial confirmada às 27/10/2026 22:11. Intervenção técnica suspensa pelo hospital pois o equipamento estava em uso clínico.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>CONCLUÍDO</t>
+          <t>VISITA REALIZADA (EQUIP. EM USO)</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -770,12 +764,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>22/10/2026 14:22</t>
+          <t>27/10/2026 22:11</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>0 min</t>
+          <t>47 min</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -785,7 +779,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>SRA. DAMARES</t>
+          <t>DR. EDUARDO COSTA</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -809,11 +803,7 @@
           <t>CONTRATO</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>[PROGRAMADA] BOTAO ANTIVANDALIMO 22MM</t>
-        </is>
-      </c>
+      <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr">
         <is>
           <t>GERAL / CORRETIVA</t>
@@ -822,7 +812,7 @@
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>FATURAMENTO 28 DDL</t>
+          <t>FATURAMENTO BOLETO BANCÁRIO (VALOR INTEGRAL) — VALOR FINAL: R$ 18,500.00</t>
         </is>
       </c>
       <c r="AH2" t="n">
@@ -830,7 +820,7 @@
       </c>
       <c r="AI2" t="inlineStr">
         <is>
-          <t>É NECESSARIO SUBSTITUIR O BOTAO DA PERA</t>
+          <t>MANUTENÇÃO PREVENTIVA PROGRAMADA</t>
         </is>
       </c>
       <c r="AJ2" t="inlineStr">
@@ -840,10 +830,7 @@
       </c>
       <c r="AK2" t="inlineStr">
         <is>
-          <t>REALIZADO SUBSTITUIÇÃO DO BOTÃO DO HANDSWITCH (PERA).
-- REALIZADO SUBSTITUIÇÃO DA GRAXA ISOLANTE DOS CONECTORES DO CABO FEDERAL DO ANODO E CATODO.
-- REALIZADO TESTES OPERACIONAIS DE FUNCIONAMENTO.
-- REALIZADO ACOMPANHAMENTO DE EXAMES COM PACIENTES OK</t>
+          <t>EQUIPAMENTO EM USO CLÍNICO NO SETOR</t>
         </is>
       </c>
       <c r="AL2" t="inlineStr">
@@ -853,21 +840,26 @@
       </c>
       <c r="AM2" t="inlineStr">
         <is>
-          <t>REALIZADO SUBSTITUIÇÃO DO BOTÃO DO HANDSWITCH (PERA).
-- REALIZADO SUBSTITUIÇÃO DA GRAXA ISOLANTE DOS CONECTORES DO CABO FEDERAL DO ANODO E CATODO.
-- REALIZADO TESTES OPERACIONAIS DE FUNCIONAMENTO.
-- REALIZADO ACOMPANHAMENTO DE EXAMES COM PACIENTES OK</t>
-        </is>
-      </c>
-      <c r="AN2" t="inlineStr"/>
+          <t>VISITA TÉCNICA REALIZADA. NÃO FOI POSSÍVEL REALIZAR A INTERVENÇÃO NA PRESENTE DATA POIS O EQUIPAMENTO ENCONTRAVA-SE EM USO CLÍNICO.</t>
+        </is>
+      </c>
+      <c r="AN2" t="inlineStr">
+        <is>
+          <t>DENTRO DAS NORMAS / HOMOLOGADO</t>
+        </is>
+      </c>
       <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>LIBERADO PARA USO NORMAL</t>
+          <t>EM USO CLÍNICO</t>
         </is>
       </c>
       <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAAEAAAABCAYAAAAfFcSJAAAADUlEQVR42mNk+M9QDwADhgGAWjR9awAAAABJRU5ErkJggg==</t>
+        </is>
+      </c>
       <c r="AS2" t="inlineStr"/>
       <c r="AT2" t="inlineStr"/>
       <c r="AU2" t="inlineStr"/>

</xml_diff>

<commit_message>
fix(v29): correcao da busca e filtros no estoque e limpeza de todos os registros de teste
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -749,12 +749,12 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>[REAGENDAMENTO NECESSÁRIO] Visita presencial confirmada às 27/10/2026 22:11. Intervenção técnica suspensa pelo hospital pois o equipamento estava em uso clínico.</t>
+          <t>[CONCLUÍDO - GERAL / CORRETIVA] Sem pendências restantes.</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>VISITA REALIZADA (EQUIP. EM USO)</t>
+          <t>ATIVO</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -764,12 +764,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>27/10/2026 22:11</t>
+          <t>28/10/2026 00:17</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>47 min</t>
+          <t>2h 53min</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -779,7 +779,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>DR. EDUARDO COSTA</t>
+          <t>SRA. DAMARES</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -788,14 +788,16 @@
         </is>
       </c>
       <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\EVIDENCIA_1_OS1_20261028_001719.png</t>
+        </is>
+      </c>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>5585996197923.0</t>
-        </is>
+      <c r="AA2" t="n">
+        <v>5585996197923</v>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr">
@@ -812,11 +814,11 @@
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>FATURAMENTO BOLETO BANCÁRIO (VALOR INTEGRAL) — VALOR FINAL: R$ 18,500.00</t>
+          <t>FATURAMENTO 28 DDL</t>
         </is>
       </c>
       <c r="AH2" t="n">
-        <v>18500</v>
+        <v>85000</v>
       </c>
       <c r="AI2" t="inlineStr">
         <is>
@@ -840,7 +842,7 @@
       </c>
       <c r="AM2" t="inlineStr">
         <is>
-          <t>VISITA TÉCNICA REALIZADA. NÃO FOI POSSÍVEL REALIZAR A INTERVENÇÃO NA PRESENTE DATA POIS O EQUIPAMENTO ENCONTRAVA-SE EM USO CLÍNICO.</t>
+          <t>TESTE DE PAYLOAD PESADO FOTOS BASE64</t>
         </is>
       </c>
       <c r="AN2" t="inlineStr">
@@ -848,13 +850,21 @@
           <t>DENTRO DAS NORMAS / HOMOLOGADO</t>
         </is>
       </c>
-      <c r="AO2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr">
+        <is>
+          <t>CONCORRÊNCIA DE ESCRITA TIMESTAMP 1793157433.7442496</t>
+        </is>
+      </c>
       <c r="AP2" t="inlineStr">
         <is>
-          <t>EM USO CLÍNICO</t>
-        </is>
-      </c>
-      <c r="AQ2" t="inlineStr"/>
+          <t>LIBERADO PARA USO NORMAL</t>
+        </is>
+      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\EVIDENCIA_2_OS1_20261028_001719.png</t>
+        </is>
+      </c>
       <c r="AR2" t="inlineStr">
         <is>
           <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAAEAAAABCAYAAAAfFcSJAAAADUlEQVR42mNk+M9QDwADhgGAWjR9awAAAABJRU5ErkJggg==</t>
@@ -1024,7 +1034,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>NETTO</t>
+          <t>ANTONIO</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1062,12 +1072,12 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>25/10/2026 23:09</t>
+          <t>28/10/2026 00:04</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>0 min</t>
+          <t>48h 55min</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -1077,12 +1087,12 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>DR ELIEZER</t>
+          <t>RESPONSÁVEL LOCAL</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>NETTO - TÉCNICO CFT</t>
+          <t>ANTONIO - TÉCNICO</t>
         </is>
       </c>
       <c r="V4" t="inlineStr"/>
@@ -1110,15 +1120,15 @@
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>FATURAMENTO BOLETO BANCÁRIO (VALOR INTEGRAL) — VALOR FINAL: R$ 0.00</t>
+          <t>PIX COM 10% DE DESCONTO</t>
         </is>
       </c>
       <c r="AH4" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="AI4" t="inlineStr">
         <is>
-          <t>- EQUIPAMENTO NÃO ESTÁ DISPARANDO.</t>
+          <t>TESTE ATUALIZACAO</t>
         </is>
       </c>
       <c r="AJ4" t="inlineStr">
@@ -1138,12 +1148,12 @@
       </c>
       <c r="AM4" t="inlineStr">
         <is>
-          <t>MANUTENÇÃO PREVENTIVA E AFERIÇÃO RADIOMÉTRICA EM EQUIPAMENTO DE RAIOS-X. AFERIÇÃO DE KVP, MA E TEMPO DE DISPARO COM MULTÍMETRO RADIOMÉTRICO HOMOLOGADO. TESTE DE REPETIBILIDADE, LINEARIDADE E RENDIMENTO DO TUBO. INSPEÇÃO DA ISOLAÇÃO DOS CABOS DE ALTA TENSÃO E NÍVEL DE ÓLEO DO TANQUE GERADOR. EQUIPAMENTO LIBERADO. | [PEÇA MANUAL: 1x CABO SPIRAL E BOTÃO ANTI VANDALISMO]</t>
+          <t>TESTE EXECUTADO</t>
         </is>
       </c>
       <c r="AN4" t="inlineStr">
         <is>
-          <t>- VERIFICADO RESISTÊNCIA DO CONTATO DO BOTÃO E TESTES DAS VIAS DO CABO SPIRAL</t>
+          <t>DENTRO DAS NORMAS / HOMOLOGADO</t>
         </is>
       </c>
       <c r="AO4" t="inlineStr"/>
@@ -1163,11 +1173,7 @@
         </is>
       </c>
       <c r="AS4" t="inlineStr"/>
-      <c r="AT4" t="inlineStr">
-        <is>
-          <t>1x CABO SPIRAL E BOTÃO ANTI VANDALISMO</t>
-        </is>
-      </c>
+      <c r="AT4" t="inlineStr"/>
       <c r="AU4" t="inlineStr"/>
       <c r="AV4" t="inlineStr"/>
       <c r="AW4" t="inlineStr"/>
@@ -1218,7 +1224,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>PREVENTIVA</t>
+          <t>CALIBRAÇÃO</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1246,22 +1252,50 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>SEM PENDENCIAS APARENTES</t>
+          <t>[CONCLUÍDO - GERAL] Sem pendências restantes.</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>ATIVO</t>
-        </is>
-      </c>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr"/>
-      <c r="U5" t="inlineStr"/>
+          <t>CONCLUÍDO</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>28/10/2026 00:22</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>28/10/2026 00:22</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>0 min</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>[OK] INSPEÇÃO GERAL DA ESTATIVA, MESA DE EXAMES E CABEÇOTE MONOBLOCO | [OK] AFERIÇÃO RADIOMÉTRICA DE KVP, MA E TEMPO COM MULTÍMETRO CALIBRADO | [OK] TESTE DE REPETIBILIDADE E LINEARIDADE DA TAXA DE KERMA NO AR (RDC 611)</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL LOCAL</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>Valfredo V. O. Netto - CFT</t>
+        </is>
+      </c>
       <c r="V5" t="inlineStr"/>
-      <c r="W5" t="inlineStr"/>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\EVIDENCIA_1_OS4_20261028_002228.jpg</t>
+        </is>
+      </c>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr"/>
       <c r="Z5" t="inlineStr"/>
@@ -1273,32 +1307,68 @@
         </is>
       </c>
       <c r="AD5" t="inlineStr"/>
-      <c r="AE5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
       <c r="AF5" t="inlineStr"/>
-      <c r="AG5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr">
+        <is>
+          <t>FATURAMENTO BOLETO BANCÁRIO (VALOR INTEGRAL) — VALOR FINAL: R$ 0.00</t>
+        </is>
+      </c>
       <c r="AH5" t="n">
         <v>0</v>
       </c>
-      <c r="AI5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>SEM PENDENCIAS APARENTES</t>
+        </is>
+      </c>
       <c r="AJ5" t="inlineStr">
         <is>
           <t>OPERACIONAL</t>
         </is>
       </c>
       <c r="AK5" t="inlineStr"/>
-      <c r="AL5" t="inlineStr"/>
-      <c r="AM5" t="inlineStr"/>
-      <c r="AN5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr">
+        <is>
+          <t>DESGASTE NATURAL</t>
+        </is>
+      </c>
+      <c r="AM5" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO E REVISÃO TÉCNICA EXECUTADA CONFORME PROTOCOLO EMED. | [PEÇA MANUAL: 1x PEC-005 - BOBINA SOLENOIDE / ELETROFREIO (ESTATIVA PORTA-TUBO / MESA)]</t>
+        </is>
+      </c>
+      <c r="AN5" t="inlineStr">
+        <is>
+          <t>DENTRO DAS NORMAS / HOMOLOGADO</t>
+        </is>
+      </c>
       <c r="AO5" t="inlineStr"/>
       <c r="AP5" t="inlineStr">
         <is>
           <t>LIBERADO PARA USO NORMAL</t>
         </is>
       </c>
-      <c r="AQ5" t="inlineStr"/>
-      <c r="AR5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr">
+        <is>
+          <t>C:\Users\vitor\OneDrive\Desktop\Sistema Emed\uploads_os\EVIDENCIA_2_OS4_20261028_002228.jpg</t>
+        </is>
+      </c>
+      <c r="AR5" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAyAAAAEECAYAAADQ0lBhAAAQAElEQVR4Aezdi3XbxqIF0FHKub49ROrB/Sjuxz0I6eHllhM+HsEwQRD8ivhvLU1IgvjM7EHWmqMB4D+KHwIECBAgQIAAAQIECIwkIICMBO0wBE4FLCFAgAABAgQIbE9AANlen2sxAQIECBAgQIAAgckEBJDJ6B2YAAECBAgQILA9AS0mIIA4BwgQIECAAAECBAgQGE1AABmNunsgnwkQIECAAAECBAhsT0AA2V6fazEBAgQIECBAgACByQQEkMnoHZgAAQIECGxPQIsJECAggDgHCBAgQIAAAQIECKxfYDYtFEBm0xUqQoAAAQIECBAgQGD9AgLI+vtYC7sCPhMgQIAAAQIECEwmIIBMRu/ABAgQ2J6AFhMgQIAAAQHEOUCAAAECBAgQWL+AFhKYjYAAMpuuUBECBAgQIECAAAEC6xfYXgBZf59qIQECBAgQIECAAIHZCgggs+0aFSOwPgEtIkCAAAECBAgIIM4BAgQIECCwfgEtJECAwGwEBJDZdIWKECBAgAABAgQIrE9Ai7oCAkhXxGcCBAgQIECAAAECBAYTEEAGo7XjroDPBAgQIECAAAECBAQQ5wABAgTWL6CFBAgQIEBgNgICyGy6QkUIECBAgACB9QloEQECXQEBpCviMwECBAgQIECAAAECgwmMFkAGa4EdEyBAgAABAgQIECCwGAEBZDFdpaIEHhawIQECBAgQIEBgNgICyGy6QkUIECBAYH0CWkSAAAECXQEBpCviMwECBAgQIECAwPIFtGC2AgLIbLtGxQgQIECAAAECBAisT0AAWV+fdlvkM4HnCHz7/lHuKf/5/ldpyn+/vz6nEvZCgAABAgQILF1AAFl6D6o/gaEFEh4SPEpJiLi9vJT30pRdSXjZ7QNMysdRMMn+y1p/tIsAAQIECBDoCgggXRGfCRA4CGQGI+GhDh+H5V9793oUTLL/b98TTFKOw8nXjmPrLQsk2Ob8TXjOa8qWPbbYdm0mQGC2AgLIbLtGxQhMLJCBW2YwTqtR7RddK/tVHvo9DifdYJJB5UO7tdHqBXJupOS8zXmTYFufv4dzKt+vHkIDCRAgML3AtRoIINeEfE9giwIZxJ3OelT7mYu38s/PW8rLfr2Xz/VfylvZlR+fpZSqPPZTDyIzqMzgMn/NTnlsX7Zai0ACRc7VnBM5N1JOz9tDa/8tr8UPAQIECEwuIIBM3gUqsF6BhbasHtgfD9QSIBI8/u/nfQEi66f87+dfJSX7+OfnIZxkv025J5y8lPr+kgw8MwBNnTMYXSi5at8hkH5On6fvrwWO7m7/KPedv8UPAQIECAwhIIAMoWqfBJYs8FL+PKp+AkLCw9HCJ3xoB5Ps/3I4uXTA15JAksFoBqUJIymXtvDdsgTuDx1VyXmb2bcE3uZ9zrlltVxtCRAgsEoBAWSV3apRBL4k8Pp76wzcEg5+LxjpTQaKOW5TMojMYDL1uTZTkjCSIoyM1FkDHea+0JGZjWofRHN5YGbY3j5n3HIepXo5j5r3+awQIDCogJ0TuCYggFwT8j2BLQnMeeYgA8gMJJuZkoSRlEv9kyCSkjCSy3bSvgxsL23ju2kE0i8p6af0V2a0Lt3PkSCaUJpSnxNvJefINLV3VAIECBC4Q0AAuQPrvlWtTWCBAt3LrzLgn2szUreUzI4kiKRcruvr/i/k7yUD2wxwE0ZSip/JBBI4UhI60i8p94SOBI6UyRrgwAQIECDwiIAA8oiabQisV+D1d9OuD+h/rzr5mwSRlISRlLru1cV6ZWYkJWEkg+CLK/vyaQKxThE6nkZqRwQIEFiagACytB5TXwJDCaxpNqAOI2+fjwJOGEm55Ja/vK+p/ZfaOsV3TeC4N3QkTObyqsxypExRd8e8W8AGBAgQuCYggFwT8j2BrQhkNqDd1gzi25+X+j7tSMlgNvcL1GHkdHYk7RdCntfL3dBRX1p1mGE7PVJV0j/ppyZ0nK5jCQECBAicF1jMNwLIYrpKRQkMKJDBYnv39SC9vWQd7/NX9DqM1LMjuZG53TIhpK1x//ucR5nlSMmsktBxv6EtCBAgsAEBAWQDnby5Jmrw/QL/lkt/mS6r/clf2oWQr3XvIXTsPm/wFzq+5mlrAgQIbEBAANlAJ2sigasC+ct/e6XMErQ/r/l9Qkh3xiceLsc63+v9oeNz/TP/cXnVGRiLCRAgsEUBAWSLva7NBC4LVJe/XuG3CVx9ISSXEq2wuQ816b7QkXOock/HQ9I2IvCogO0ILEZAAFlMV6kogUEFqkH3voSd94WQXE605RDyeOjIPTZv/mHAJZz46kiAAIHxBdYXQMY3dEQCaxPY5v0g6cXzIWRXMhjPOmsvaWdCV/59lMON5OdaXZVd+VHqp1e9lVzOlhv9z61tOQECBAgQ2AsIIHsEvwQ2L7Arfx8ZZBB6tOC2D6tYKyEkA+puYzIYX6NL2pRyT+iIT0oCR7yEju7Z4jMBAgQIXBAQQC7g+IrAZgT+KC7BKq2fDKgzwG4t+ny7lhCSwJGS0JE2peRys89G9v6nKvFISeiIT0rvqhZOJOCwBAgQWIyAALKYrlJRAiMKbPWxvG3iDLDzj+J1H9NbD9bbay7rfZ7ulTakCB3L6ju1JUBgpgKqda+AAHKvmPUJrFEgg+12u17Kn+2Pm36fv/h3Q0hmDpaGUs947PYzGe8Xql7PdCR4pd05L1IubOArAgQIECBwr4AAcq+Y9c8K+GLxAtXiWzBUA17Kj86uX8tSQkgdPD5KPePRacbnx6rUl1a9uIn808N/CBAgQGBgAQFkYGC7J7BQge0+CauvwzILkEH68XevJZczHS+b6tPpcY+Dx2l/5ulV7ZmO0z1YQoAAAQIEBhEQQAZhtVMCCxTwJKzLndYXQl7K+yxDSIJRPeNxGjxyOVmCR55edbnFviVA4CYBKxEgcK+AAHKvmPUJrFXAk7Cu92xCSGYO2mvOKYQ0sx6pU7uO9fvmUqu3+qP/EiBAgACBaQSeFkCmqb6jEiAwmIAnYfXTZuagL4Rk8N+/xfBLc+zck9I/63EIHglQw9fGEQgQIECAwEUBAeQijy8JLELgOZXsDk49Ceu8a18IyeA/QeD8VsN8c+lyqwSl5mlWwxzdXgkQIECAwN0CAsjdZDYgsGqBatWte2bjEkJyP0V7nwkh7c9Dvk/w+Pb93GN1q88nW9V1HLIW9l0QECBAgMC9AgLIvWLWJ7Adgb4bmLfT+ltamtmFbgjJpVC3bPvoOpllyTGu3efRndF69Hi2I0CAwFwF1GuxAgLIYrtOxQkMINB9EtYAh1jdLl/KOP9GSBM86lmW03DocqvVnVoaRIAAgbUKCCDL71ktIPA8ge6TsDLofd7e17mnzDQM/W+E5HKry8Hjpbjcap3nl1YRIEBghQICyAo7VZMIEBhL4Ndx+kJILpH6aoDL9tcutxI8fnWCFwIECBBYioAAspSeUk8CYwhkIN0+zq68tz96f0EgdrkMqr3Ko48yboJH/6xHVTLjkvtPcsz28bwnsCUBbSVAYLECAshiu07FCQwmUA2257XvuDsb8cijjDPj0R88SknAETzWfhZpHwECBGYv8NUKCiBfFbQ9gXULnN7svO72PqN17QD3WjKbcctec59HHqtbSp959Tnr0Q04xQ8BAgQIEFiegACyvD5T49kIqAiBHoHuU7F25b1nrcOiBJTMeuSekcPS5l31GTzMejQeXgkQIEBgBQICyAo6URMIPFWgO4DOAPmpB1j5zur7MqpWK/tmNMrnzEiCh8utWlR3vLUqAQIECCxWQABZbNepOAECsxW4FuJyudXl4OGxurPtXBUjQIAAga8KCCBfFbQ9gbUJ1H/BP7Tq0Sc5Hfbg3e7XZViZTcqsx6XLrdzn4XwhQIAAgZULCCAPd7ANCWxE4JEnOW2E5mwz6xBXtb5/LQke/bMelfs8WlLeEiBAgMDqBQSQ1XexBhJ4SKB6aKuxNlrCcbqXYfU93cpjdZfQk+pIgAABAk8WEECeDGp3BFYo0H8T9QobOmKTqs9ZD5dbjUjuUM8SsB8CBAh8VUAA+aqg7QmsUWBX/j5qVu5dOFrgw0WBw03m3dXq4OGxul0XnwkQIEDgusBq1hBAVtOVGkLgiQJ/lKr4uV8gQS33evTfZF7vr74/pH7vvwQIECBAYIMCAsgGO33xTdaA8QU8Ceu6+WHW49Ila5e+u34MaxAgQIAAgRUICCAr6ERNIPB0ge5f6T0J6zLxuVmP3GT+Ut6ONs4sydGCZX1QWwIECBAg8FUBAeSrgrYnsF4Bl2Fd69uEiYSP0ydcVSXBIzeZd8Pc7te/CXJt374nQIDAsYBPBFYjIICspis1hMCgAi4d6vKeu+Qqsx6nN5lXrc1fS4JLa4G3BAgQIEBgSwLLCyBb6h1tJTClgCdhndfPrEffjebNrEd3y5fyo7vIZwIECBAgsFUBAWSrPa/dBK4J9DwJ69omq/8+Mxffvu/27ezOCFUl4aN7udV+xd5fN/X3slhIgAABAtsQEEC20c9aSeDrAlsfNB8uuTq27L/k6nid7ifhrivi83UBaxAgQGA1AgLIarpSQwg8WaD71/ytPgmrnvX42M9wvJ8IZ9YjN5qffGEBAQIECKxHQEueLSCAPFvU/gisS6BqNWd7N08fZj1OL7n65+dL6Ya0FtbR263PHh1h+ECAAAECWxcQQLZ+BtzRfqtuUKB78/RuQ4+QPXej+a78KHnK1QZPB00mQIAAAQLPEBBAnqFoHwTWKlD/hb9qNe+1ZFagtWB1b5tLri792x5fbXTtes9erEuAAAECBFYjIICspis1hMBAAt1ZkL7Hzw506NF3m3C1Kx/74x5fcrX7NeshOOxp/BLYmoD2EiDwbAEB5Nmi9kdgbQIZdGcA3m5XBurtz0t/38x69IWrZ9xovtUb+Jd+Xqg/AQIECAwicHMAGeTodkqAwDIEuk96ykA9g/Zl1P5yLdOOvlmPUqqS8JEAVvwQIECAAAECzxIQQJ4laT8EhhOYx567syC7cvpY2nnU9PZaZCanDh/H26StudF8mPBRHR/MJwIECBAgsC0BAWRb/a21BB4XqGdB2oPn5T6WN7Me/U+5qj5nPeq2Pm5lyxUJaAoBAgQIPFtAAHm2qP0RWLNA94b03QJnQQ6zHsc3mueSq+FmPQ7H2pW/13yKaBsBAgSeJmBHqxUQQFbbtRpGYACB+pKkqrXnZT2Wt3/Wo5TmkqtWw572NrMtT9uZHREgQIAAgeULCCDz70M1JDAvge4syBJuSE8I+PZ9t4c8zETsP+x/q5IbzYe85OrfcnzMP0pV/BAgQIAAgQ0LCCAb7nxNJ/CQQGZBMmPQ3nhX3tsfZ/X+cMnVcbXShquXXB1v8tCn7iN44/fQjmxEgAABAgTWISCArKMftYLAuAL1jEHVOuj8bkivZz0+9jMcp+Fo6FmPFsz+bXsGpG22/8ovAQJnBXxBgMBqBQSQ1XathhEYNp+88AAAEABJREFUWKB7KdZuRrMgCR/143Xbg/+AVOWfny9lrFmI1CNHbYob0BsJrwQIECAwY4GhqyaADC1s/wTWKlAP4qtW8+ZxQ/q1S65aFR78rfs/Bid2AAIECBBYnoAAsrw+U+PRBBzoqkB3FmTqG9ITPlKH44pXZdxLro6P3v5Uh7b2Eu8JECBAgMDmBASQzXW5BhN4okAG1Lvy42iPu4kuxToXPsa40fwIoPXhOAxVrW+8vSbgewIECBBYrYAAstqu1TACIwnM4Yb03GtxPNgvJcEo4WMkhquHcf/HVSIrECAwDwG1IDC0gAAytLD9E9iCQPdSrF15H7XZp8erSh2MRq3G0cEyI3O0wAcCBAgQIEAgAgJIFHqLhQQI3CyQS7FKqcrhZ7wb0uuB/vHTruY089GYTB2Imnp4JUCAAAECEwsIIBN3gMMTWI1Adxake0nUPQ29dd2Ej+5xcsP5rdsPuV63XkMey74JECBAgMCCBASQBXWWqhKYtUBmQXLfRbuSCQjtz898n313B/k5furxzOM8Y1+p1zP2Yx8ERhBwCAIECAwtIIAMLWz/BLYk0L3MKAEhN4g/2+Bc+Oge/9nHvXV/qd+t61qPAAECBAjUApv5rwCyma7WUAIjCXQvgdo9+Yb0BJoEm3ZzMsMwl/DRrlfzfs51a+rolQABAgQIjCQggIwE7TB3CFh12QL1JVBVqxGvJaGhteBLb3fl42j7Xfkx+ROvjiq0//BS/tz/1y8BAgQIECDQIyCA9KBYRIDAFwW6N6R3Q8Oju//2/aOz6fSP2+1U6NfHw1O5dvuA9GvhEl7UkQABAgQIDC0ggAwtbP8EtihwOgtSylfvi6i3Pwzs4zrHx+3W9UztFAIECNwjYF0CmxEQQDbT1RpKYGSBbjjIfRuPXoqVQX22bzehe69J+7sp33fr6f6PKXvDsQkQIEBghgLzCyAzRFIlAgQeFOhefrQr73fvqS98ZL/1LMvduxt0g9S1fYDUs/3ZewIECBAgQKAIIE4CAgR+Czz9Tf3X/6q13/tuSM+MSXdGIYP6er+t3c7gbcJHt65zrOcMqFSBAAECBLYtIIBsu/+1nsDwAqc3pN8+C9K9eX2u4aNPMXXtW24ZgX4BSwkQILAZAQFkM12toQQmEqgvlTqeBclswbXqLOeJV/UN9u3Zj4QPsx/Xetj3BAgQmImAaowtIICMLe54BLYo0J0FyWA9l1eds6gDyvyfeNXUP+1p3nslQIAAAQIELgoIIBd5tvWl1hIYTCCzIJkVaB9gd+aG9ISP7oB+rk+8SntS37w2Je00+9FoeCVAgAABAicCAsgJiQUECAwiUA/Kq9a+T29Iz2C+Gz4yoE+AaW04q7fd+tbtvLeK1idAgAABApsREEA209UaSmAGAt1LsXatWZBcktUdzCd8zHlA371PJfWdAbMqECBwj4B1CRAYW0AAGVvc8QhsWaCeyahaBK8lsx5ZsLQnXtXh4/g+lTmHpRgrBAgQIEBgBgK/A8gM6qIKBAhsQaA7C5JZj3ow3259VeY6mM9Mzbfvu31lj8OH2Y89iV8CBAgQIHBdQAC5bmQNAkMLbGv/mQU5HawfD+b/+fk2S5SEj+5MTSqam+TnGphSP4UAAQIECMxIQACZUWeoCoHNCFwarGcwP0eIXCp2LnwkVM2xzup0g4BVCBAgQGBsAQFkbHHHI0CgFjidBSkly+Y4mE/4yKVidc2b/1YlYWmO9W1q6JUAAQJzFlC3zQoIIJvteg0nMKFA/4C+lD9KVeb201/XquQyMeFjbr2lPgQIECCwAAEBZPpOUgMCBBqBvkucmu+meO0LH5mlSfiYoj6OSYAAAQIEViAggKygEzWBwOIETi9nOjQhg/7Dp4Hfndl9bjbPk7m69Uz4uHT/ypndWUyAAAECBAgcBASQg4V3BAiMIdANGBnUt4+bQX8CQHvZmO9Tv3om5vjJXKmn8DFmTzjW2gW0jwCBzQoIIJvteg0nMBOBDOozuG9XZ1fe2x9HeZ/Q0zfrkYOnfqln3isECBAgQGDhAlNXXwCZugccn8DWBDLDcWhz9fm2HtzX7z8XlNeSQFBG+jk361FK9fmkq7p+xQ8BAgQIECDwdQEB5OuG9rBYARUfXaAbKnbl7991eCk/fr/Pm90IsyCpz6VZj9xs7klX6Q2FAAECBAg8TUAAeRqlHREgcFXg33J8X0X7sbv1QL8qh5/XkpmJw+fnvsu+++71MOvxXOdze7OcAAECBDYrIIBstus1nMAEAi/lz6Oj1qHjsKg7C5LLtTJLcVjj6++yP7MeX3e0BwIEFiug4gSmFhBApu4BxyewLYHDDEhu7O62PYGku3xXnndDulmPrrjPBAgQIEBgdIENB5DRrR2QwLYFMvi/RaC+4btqrfr1G9LNerQ4vSVAgAABAtMKCCDT+js6gW0KpNV10Mi709K9FCv3aiREnK55fUmCT7Yv5TD7Uj5/qvJS3sqlenyu5j8ECBAgQIDAMwUEkGdq2hcBAucFcj/H4dvq8LbnXS7Fys3g7a8SIu4JIVnXvR5tQe8JfAr4DwECBKYWEECm7gHHJ7AFgYSBdjvbj99tL2+/zyNwHw0hZj3akt4TIECAwDwE1OKXgADyC8ILAQIDClx6/O6lw94bQhJ0zHpcEvUdAQIECBCYXEAAmbwLNlgBTd6ewLXH714SuTWEmPW4pOg7AgQIECAwGwEBZDZdoSIEVi1wuAG8+5jdW5p9LYSY9bhF8XMd/yFAgAABAlMLCCBT94DjE1i7QGYmntHGcyHk2/fdfveHgLP/sP+tiidc7Rn8EiAwIwFVIUDgl4AA8gvCCwECIwl85bG3dQi5XNHMsGS9+klal9f1LQECBAgQIDC6wPgBZPQmOiABApMK3PP43VsqmoBxbj2zHudkLCdAgAABArMREEBm0xUqQmB4gdGP0L386pbH716qZPZ3HGgure07AgQIECBAYIYCAsgMO0WVCKxW4I9SlUd+6sfr7sq18LEr74/s3jYERhBwCAIECBD4JSCA/ILwQoDAAAJfefxuqlMHj4+yKx/52ClV2ZUfnWWvJU/E6iz0kQABAgS2LKDtcxMQQObWI+pDYL0C1c1NOw4e3Sdclc/gkRvNc0N77vs43rEQcuzhEwECBAgQmJWAADKr7hi2MvZOYBECuc+jnvE4DR6lVOWfny8lwaP8+snTroSQXxheCBAgQIDA/AUEkPn3kRoSWItAX6A4tK2e9Th3n0dVEjIy63HY4vBu/iHkUFfvCBAgQIDAxgUEkI2fAJpPYFCBW556VQePj1LPenSrU/0OHgkZ3W/bn/N9Qkp7WSkuxyp+CGxdQPsJEJibgAAytx5RHwJrFkjYaNqX97lhvA4ep7MjucE8Mx4JFs02116zrhByTcn3BAgQIEBgHIEzRxFAzsBYTIDAEwT6HrubezwuBY+++zzuqYoQco+WdQkQIECAwOgCAsjo5A64QQFNbgQy21H/Wx6nMx4JHpm9yKxHs/6jr0LIo3K2I0CAAAECgwsIIIMTOwCBDQv8W/qCRun83H6fR2fDix+FkIs82/lSSwkQIEBgbgICyNx6RH0ILF2gubfj2/dzT7RqWjhM8Gj2nlchJAoKAQIEphFwVAJnBASQMzAWEyBwp8D1ezuywyZ0vJRcapWAkKVDlhwjl3YdH8PTsY49fCJAgAABAqMJCCDDUzsCgfULZNbj/L0dx+1PIDheMvynHFMIGd7ZEQgQIECAwA0CAsgNSFYhQOAhgarsyo/9ltW+TPTbOmxCSF2f1sJiJqT4IUCAAAEC4woIION6OxqBdQocBvcJG1XJbEMusfrfz786DX4tmS3pLBztY+ojhIzG7UAbF9B8AgQInBEQQM7AWEyAwJ0CGdwndKQkkDSbv5TMgjSfSrntyViH9Z/9LvXsCyG5h+XZx7I/AgQIECAwgcDcDymAzL2H1I/A0gXaYSRteSl/5mXS0hdCcg+LEDJptzg4AQIECGxDQADZRj9vtJWaPSOBqlWXaS/DaioihDQSXgkQIECAwKgCAsio3A5GYKMC3cuwduV9FhJCyHDdYM8ECBAgQOCMgAByBsZiAgSeKFBfhlW19jiPWZBUSAiJgkKAwIoENIXA3AUEkLn3kPoRWItAdxZk6pvR265CSFvDewIECBAgMKjAigPIoG52ToDAvQL1LMhhqzncjH6oTSlCSFvDewIECBAgMJiAADIYrR0T2LDA+abP8zKspr5CSCPhlQABAgQIDCYggAxGa8cECJwIdC/D2s3kZvR2RYWQtob3CxRQZQIECMxdQACZew+pH4E1CdSXYVWtJs3nZvRWpVyO1cbwngABAgRuFLDajQICyI1QViNA4EkCS5gFSVPNhERBIUCAAAECTxcQQJ5OaocFAYFLAvUsSHuN1/aHWb0XQmbVHSpDgAABAusQEEDW0Y9aQWBZArvy46jC375/HH2e04eFhZA50akLAQIECBDoExBA+lQsI0BgWIE/Svs+kLL/eS3/+f7X/nWev0LIPPtFrQjMS0BtCBC4UUAAuRHKagQIPFEgl2HtOrMgL+VdCHmisV0RIECAAIGZCjw/gMy0oapFgMDMBJY4q7DEOs+s21WHAAECBAgIIM4BAisSWFxTzg3o//vdjemL60wVJkCAAAECtwkIILc5WYsAgaEE+kLIrnwUIWQocfsdRsBeCRAgQOBGAQHkRiirESAwoEBCSCnHN6bvynuZ80/qvLT7WObsqW4ECBB4WMCGSxMQQJbWY+pLYK0C//x82zet2pfm97XM+fG8qaUQEgWFAAECBAjcJSCA3MU175XVjsDiBV46T8Yq5XXWT8Yq+x8hZI/glwABAgQI3C4ggNxuZU0CBIYWyON5X8rb0WHm/njeVPZ/P/8qLseKhEKAAAECBK4KCCBXiaxAgMCoAgkhSxzMmwkZ9TRxMAIHAe8IEFiagACytB5TXwJbEDg3mJ/zk7HSL+fq/Z/vf+VrhQABAgQIrErgwcYIIA/C2YwAgYEF+gbzc388b0j66r2Ey8hSd4UAAQIECIwgIICMgOwQqxfQwKEEMpg/fTzvvP+NkFik3ku8jCx1VwgQIECAwMACAsjAwHZPgMAXBU4fz1vKrrx/ca/Db54Q0g1PZkIGcLdLAgQIEFiagACytB5TXwJbFKhDSLvlr7P/N0JS27reVd7+LkLIbwpvCBBYuIDqE3hQQAB5EM5mBAiMLNB9PO8S/o2QEAkhUVAIECBAgMBvAQHkN8XDb2xIgMAYAnk8bzeEZDbh2/fd7P+xwnMhZO5P9RqjXx2DAAECBDYnIIBsrss1mMCCBRJCjm7u/tWWBJG5P+q2L4Qs4alev4i9ELhbIAE7Jf9vpty9AxsQILBWAQFkrT2rXQTWKpCbu8+FkLnPhgghaz0rt9muvlYncKR8+/5RErBT8geClCzv28YyAgQ2JyCAbK7LNZjACgQSQv75+bIf4Pw4aU0GOnMOIk8rQTwAAA3NSURBVELISZdZsHCBBIuUdujIPVrdZv1bXosfAgSeIrD0nQggS+9B9SewZYEEkb7ZkJjUQeRjlveHCCHpIWXpAreEjqW3Uf0JEBhEQAAZhNVOxxFwFAJ7gYSQc7Mh+Stsgsgcrz8XQvad53dxAk3oyCxjLq/K/2PnG1EdffVS/jz67AMBApsVEEA22/UaTmBlApeCSEJIBkxzCyJLDiErO30054LAvaEjT6vLHwX6zu8Lh/EVAQLbERBAttPXWkpgGwIJIhkA9V2aNccg0jdIy1+WM+jbRo9p5RwFcv7lno4E95yP12Y68v9cEzrytLr+NrkHpN/l7qU2ILB0AQFk6T2o/gQInApkAJQg0hdCsnaCSGZDUvJ56iKETN0Djh+BYUJH9qwQIEDgSGDBAeSoHT4QIEDgVCAhJH+V7QsiCSEpQsipmyXbERg6dOzK30eYOd7RAh8IENiigACyxV7XZgJfFVja9teCSC4zmUMQMROytDNrmfVNCLj38qr6Equ3ktnFe1r9Rzm+Eb34IUCAQCkCiLOAAIHtCCSIZDYkpdvqzIbMIYgIId2e8bkj8NDHr4aOe4PHQ5W0EQECWxEQQLbS09pJgEAtkBCS0hdCskaCSGZDMmDL5ynKSzn9BxZzI3DqlTJFnRxzeQI5h78y0zFE6PCPES7vPFLjtoD3TxIQQJ4EaTcECCxMICHk0v0hzYB/imZl4JdLXrrHTjhKSQhJ6X7vM4FD6PgoOYdveXpVzrXMvOW8S3mm4rP398y62RcBApMJCCCT0S/4wKpOYE0C14LIVJdlZeCWgWGfdUJIylR166uTZdMJ9IeOc4+8rfYVrUrOraFCx/4AZ3/9Y4RnaXxBYEsCAsiWeltbCRA4L5AgUl+WVZ2sNNVgPyGkM0szm7qdVMSCUQW+Ejqa4DFehU//nxrv2I5EgMAMBQSQGXaKKhEgMJFAQkgGZ3UQOa1EgsgUlz7V9XopqVfKac3K/i/a78WMSFn1T0JHzr/c13G4vOq2mY6c1wm0YwOlzseXgZ2r79g1e+R4tiFA4EkCAsiTIO2GAIEVCbQH/N1mJYRMNdBPvVJy+cwtQaQe/HVb4POSBNKHKU3oyPl3PKDvtqbah9G3ksCRMkXoSI3adc5nhQABAi2B+wNIa2NvCRAgsGqBDPbPXQKVgWATRDLYGhMig8pLdUtdUr/8lTx/MU/JMmUZAjmfUprQkX68LXS8fAaPnB9TtbRd7746nwvOU9XXcQkQmERAAJmE3UEJPCZgq4kEMtg/N3BqBvpNGBl7sJ+6nQtJ4Ur9Upr6ZZkyP4EM3FOWGDqi2a57X/AopZ6Zyfla/BAgsHUBAWTrZ4D2EyBwm0AGTpcG+tlLBvopzWB/zDBya/2auqW+yj0Cw6zbHrgvaaajrZHz/Hzd6+Ax5eVg7bp6T4DALAQEkFl0g0oQILAYgVsG+mlMgkhKBvz5q3YGaRls5rshS7t+l2ZtUq/Uaci62He/QM6DnBPpg/MD92bbZgA//eVVTY2a15w/aUPO82bZ4bWp91uZ8pKwQ328W7SAyq9NQABZW49qDwEC4wjcMtA/1OS1ZJCWwWYGbBm4pRy+f/671C8lISSl7wipU1Ofvu8te57AWkJHRHLu5rzJ+ZPP3ZLzzYxHV8VnAgRaAgJIC2Pub9WPAIEZCmSQn5LLsw5Pp6ou1jQDt5QM4jKYS7m4wRe+TN1SUr8MDPt2NVZd+o69xmUJGynp1zXMdDR9lDalPTlfmmXt15xfOc9yvrWXe0+AAIGOgADSAfGRAAECPQK3LcqlJhl85a+/GYhlQJZyaesM5lISRjK4y6A1A71L2zz6XV23+t8T6dtH6pGSOqT0rWNZLZA+SolT+q0uu89/iyUzXSmx7L8hu95Hc2N2zpWcMzl/mm/m9Jp2pn1pU197co6nDTm/5lRvdSFAYLYCAshsu0bFCBBYvEAGZCkZnB1mRy41a5xLtZo6ZeDYV5sMnFMSijLA7ltnC8sy8E6JQQbgdTkXMl5vJKlKzoWcE3MOHWlM2p42nwseCVBpR86nrD9YsWMCBNYmIICsrUe1hwCBeQrkr9sZqGXAllIP/quLlU0ISEkQyEAwA+GLG9z5ZVOfS3Vpjv/sY99Z1cFWzyA7Je2LcV2+GjK61a0+Q0cdPOZ/U3Y84nApeDRt6bbUZwIE1iUwUGsEkIFg7ZYAAQIXBerB/1tpwkgdAi5t8rofxL5/XuKTQJIBcwaKl7a49bumLqlDSt92Sw4icUqJWQbWdXl+yMiMQPwyOG9K+reZ6UgI7bOdy7IYxeaW4DH3tszFVD0IEOgVEEB6WSwkcCTgA4FhBRIAUjJYzcA1g9gMZi8dNYEgA8UmjGRwfWn9W75LHVJSj7oOp1vluM885ukRHluSwXNKHDKIrsu4ISNBI34ZnDflsdaMu1Xc4pXzqe8ej5yLOS/TvrRr3No5GgECKxQQQFbYqZpEgMCCBTLAyyA2g70mCJwLA00zEwpSEgwykMwgPIPK5vtHXus6zOCG9Vbl06aUtC/trIuQ0SK6620sYyh43MVmZQIEvi4ggHzd0B4IECAwnECCQMqtYSR/wU4YyaCyCSQZZD5aXsqf+8ZV+9L/m2OlPONY5+soZPTrP740IS7nSM6X071UxYzHqcoWl2gzgYEEBJCBYO2WAAECTxdIEElJGMkAsZ4Zqa4c53X//TPKfjdXf59xnL59XD1wzwpxqcqu/Cixakrs6tmltxLLzDg1pWcnq1uU4JGwmNB42rjq0yo+MTn93hICBAg8RUAAuc5oDQIECMxPIAPEDKAzWMygOgPtlPnVdMgaVfudV0LGXuHar+BxTcj3BAiMKCCAjIjtUAQI3Ctg/ZsFEkZSjsNIPUDPTcTDl5urul/x/nrtipmMPdzdv819Hv0zHuUzvCXEJtDevXMbECBA4DEBAeQxN1sRIEBgvgIJIikZWI5Xzt+wfirVXGaVAfDf+0Hw3+Wl/CiX6pr2ZJDclNN9WtIWaILHufs8EugSVuPa3q793nsCBAgMJCCADARrtwQIENicQAazGdRmcHtb419L/jKfkoFy7k2oy0fJDem5bCglg+nb9metWMUunn03mKdv0kfpK1oECMxWYO0VE0DW3sPaR4AAgbEFMrjNIDeD3frSr3tr8Lrf4PVsOEkoaUoG3PuVN/8bh0vBI/2QG/HTN5vHAkCAwNQCAsjUPeD4FwR8RYDAogUy2K0vq3rZh4m3kkDSlAyIH2vcIZi8lPeSv/TXsyZ5VO9HaYJJXjMoLwv8Sb3bJW1JScA4LmlzXeLQN+MR5wSP9EMuX1sghyoTILA+AQFkfX2qRQQIEPi6wLP3kMFvAklTMiDOLElKBshNMMlrBs2PHf+2cNIM7h87xn1bNcdqXhMkUo6DxEc5hKjdZ6hKoGhKglZKHTBe9xVoyv7t2d/qM/TFOfZnV/MFAQIExhcQQMY3d0QCBAgQaAtkgNwEk7xm0JxgktIOJ3Uwqdqb3vH+dT8gf/8szcD+MOj/+D1zkqBwaaf5vikJEk05DhT1rET23xyreU2QSLkvTFyqUfe7at/Gt88b+uPa/dbnRQioJIG1Cwgga+9h7SNAgMCSBTKITihJqYNJBtcv+wH28WVddTh5tKXH4STBoS4f+5mJlP5AkSDRlONA8Wg9bt2u2q9Yl8wYNSVhLUYx26/glwABAnMVmHEAmSuZehEgQIDALAQy0E4wScnAOzMmKRmIpzQD88fDyeu+nSn7l8F+6yBR17Equ/Ljs6T+7ZJ2HUpCWF3S9qbEY7Bq2jEBAgSeJyCAPM/SngisR0BLCCxZIAPxlGZg3g0nzSA/r/XA/1mt/VqYSD2bOqf+7fKsGtoPAQIEZiAggMygE1SBAAECBEYSyKC+GeTnNYP+ZmYhMw4JJU2pw0kdKpplec16TWm2rV/rWYl6n28l+0/JMdvlSlN9TYAAgbULCCBr72HtI0CAAIHbBBISEhia0gSJvDbL8pr1mnLbnq1FgMAyBNRyJAEBZCRohyFAgAABAgQIECBAoBQBxFlwKmAJAQIECBAgQIAAgYEEBJCBYO2WAAECjwjYhgABAgQIrF1AAFl7D2sfAQIECBAgcIuAdQgQGElAABkJ2mEIECBAgAABAgQIEOi7B4QKAQIECBAgQIAAAQIEBhIwAzIQrN0SeETANgQIECBAgACBtQsIIGvvYe0jQIAAgVsErEOAAAECIwkIICNBOwwBAgQIECBAgECfgGVbExBAttbj2kuAAAECBAgQIEBgQgEBZEL87qF9JkCAAAECBAgQILB2AQFk7T2sfQQI3CJgHQIECBAgQGAkAQFkJGiHIUCAAAECBPoELCNAYGsCAsjWelx7CRAgQIAAAQIECERgoiKATATvsAQIECBAgAABAgS2KCCAbLHXtbkr4DMBAgQIECBAgMBIAgLISNAOQ4AAAQJ9ApYRIECAwNYEBJCt9bj2EiBAgAABAgQioBCYSEAAmQjeYQkQIECAAAECBAhsUUAAKWWL/a7NBAgQIECAAAECBCYREEAmYXdQAgRqAf8lQIAAAQIEtiYggGytx7WXAAECBAhEQCFAgMBEAgLIRPAOS4AAAQIECBAgsE2BrbdaANn6GaD9BAgQIECAAAECBEYUEEBGxHaoroDPBAgQIECAAAECWxMQQLbW49pLgACBCCgECBAgQGAiAQFkIniHJUCAAAECBLYpoNUEti7w/wAAAP//tRbznwAAAAZJREFUAwDmmnTb76D/AgAAAABJRU5ErkJggg==</t>
+        </is>
+      </c>
       <c r="AS5" t="inlineStr"/>
-      <c r="AT5" t="inlineStr"/>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>1x PEC-005 - BOBINA SOLENOIDE / ELETROFREIO (ESTATIVA PORTA-TUBO / MESA)</t>
+        </is>
+      </c>
       <c r="AU5" t="inlineStr"/>
       <c r="AV5" t="inlineStr"/>
       <c r="AW5" t="inlineStr"/>
@@ -3480,10 +3550,8 @@
       </c>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr">
-        <is>
-          <t>5585996197923.0</t>
-        </is>
+      <c r="AA22" t="n">
+        <v>5585996197923</v>
       </c>
       <c r="AB22" t="inlineStr">
         <is>
@@ -3659,10 +3727,8 @@
       </c>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="inlineStr">
-        <is>
-          <t>5585996197923.0</t>
-        </is>
+      <c r="AA23" t="n">
+        <v>5585996197923</v>
       </c>
       <c r="AB23" t="inlineStr">
         <is>
@@ -3834,10 +3900,8 @@
       </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr">
-        <is>
-          <t>859858585858585</t>
-        </is>
+      <c r="AA24" t="n">
+        <v>859858585858585</v>
       </c>
       <c r="AB24" t="inlineStr">
         <is>
@@ -4005,10 +4069,8 @@
       </c>
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="inlineStr">
-        <is>
-          <t>859858585858585</t>
-        </is>
+      <c r="AA25" t="n">
+        <v>859858585858585</v>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
@@ -4196,10 +4258,8 @@
           <t>radiologia@imediata.com.br</t>
         </is>
       </c>
-      <c r="AA26" t="inlineStr">
-        <is>
-          <t>87988881234</t>
-        </is>
+      <c r="AA26" t="n">
+        <v>87988881234</v>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
@@ -4391,10 +4451,8 @@
       </c>
       <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="inlineStr">
-        <is>
-          <t>34684651654</t>
-        </is>
+      <c r="AA27" t="n">
+        <v>34684651654</v>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
@@ -4566,10 +4624,8 @@
       </c>
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="inlineStr">
-        <is>
-          <t>5585996197923.0</t>
-        </is>
+      <c r="AA28" t="n">
+        <v>5585996197923</v>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
@@ -4737,10 +4793,8 @@
       </c>
       <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="inlineStr">
-        <is>
-          <t>8598598712165</t>
-        </is>
+      <c r="AA29" t="n">
+        <v>8598598712165</v>
       </c>
       <c r="AB29" t="inlineStr">
         <is>
@@ -4896,10 +4950,8 @@
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr"/>
       <c r="Z30" t="inlineStr"/>
-      <c r="AA30" t="inlineStr">
-        <is>
-          <t>9896659858</t>
-        </is>
+      <c r="AA30" t="n">
+        <v>9896659858</v>
       </c>
       <c r="AB30" t="inlineStr"/>
       <c r="AC30" t="inlineStr">
@@ -5059,10 +5111,8 @@
       </c>
       <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr"/>
-      <c r="AA31" t="inlineStr">
-        <is>
-          <t>8678198733</t>
-        </is>
+      <c r="AA31" t="n">
+        <v>8678198733</v>
       </c>
       <c r="AB31" t="inlineStr">
         <is>
@@ -5234,10 +5284,8 @@
       </c>
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
-      <c r="AA32" t="inlineStr">
-        <is>
-          <t>85987654689</t>
-        </is>
+      <c r="AA32" t="n">
+        <v>85987654689</v>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
@@ -5651,10 +5699,8 @@
       <c r="X35" t="inlineStr"/>
       <c r="Y35" t="inlineStr"/>
       <c r="Z35" t="inlineStr"/>
-      <c r="AA35" t="inlineStr">
-        <is>
-          <t>8898654682</t>
-        </is>
+      <c r="AA35" t="n">
+        <v>8898654682</v>
       </c>
       <c r="AB35" t="inlineStr"/>
       <c r="AC35" t="inlineStr"/>

</xml_diff>

<commit_message>
feat(v37): baixa automatica de pecas no fechamento da OS, quarentena fiscal de 24h e emissao de remessa para diagnostico CFOP 5915 e 6915
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BA35"/>
+  <dimension ref="A1:BA41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -796,8 +796,10 @@
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr"/>
       <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="n">
-        <v>5585996197923</v>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr">
@@ -814,11 +816,11 @@
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>FATURAMENTO 28 DDL</t>
+          <t>PIX COM 10% DE DESCONTO</t>
         </is>
       </c>
       <c r="AH2" t="n">
-        <v>85000</v>
+        <v>450</v>
       </c>
       <c r="AI2" t="inlineStr">
         <is>
@@ -3550,8 +3552,10 @@
       </c>
       <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="n">
-        <v>5585996197923</v>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
       </c>
       <c r="AB22" t="inlineStr">
         <is>
@@ -3727,8 +3731,10 @@
       </c>
       <c r="Y23" t="inlineStr"/>
       <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="n">
-        <v>5585996197923</v>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
       </c>
       <c r="AB23" t="inlineStr">
         <is>
@@ -3900,8 +3906,10 @@
       </c>
       <c r="Y24" t="inlineStr"/>
       <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="n">
-        <v>859858585858585</v>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>859858585858585</t>
+        </is>
       </c>
       <c r="AB24" t="inlineStr">
         <is>
@@ -4069,8 +4077,10 @@
       </c>
       <c r="Y25" t="inlineStr"/>
       <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="n">
-        <v>859858585858585</v>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>859858585858585</t>
+        </is>
       </c>
       <c r="AB25" t="inlineStr">
         <is>
@@ -4258,8 +4268,10 @@
           <t>radiologia@imediata.com.br</t>
         </is>
       </c>
-      <c r="AA26" t="n">
-        <v>87988881234</v>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>87988881234</t>
+        </is>
       </c>
       <c r="AB26" t="inlineStr">
         <is>
@@ -4451,8 +4463,10 @@
       </c>
       <c r="Y27" t="inlineStr"/>
       <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="n">
-        <v>34684651654</v>
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>34684651654</t>
+        </is>
       </c>
       <c r="AB27" t="inlineStr">
         <is>
@@ -4624,8 +4638,10 @@
       </c>
       <c r="Y28" t="inlineStr"/>
       <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="n">
-        <v>5585996197923</v>
+      <c r="AA28" t="inlineStr">
+        <is>
+          <t>5585996197923.0</t>
+        </is>
       </c>
       <c r="AB28" t="inlineStr">
         <is>
@@ -4793,8 +4809,10 @@
       </c>
       <c r="Y29" t="inlineStr"/>
       <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="n">
-        <v>8598598712165</v>
+      <c r="AA29" t="inlineStr">
+        <is>
+          <t>8598598712165</t>
+        </is>
       </c>
       <c r="AB29" t="inlineStr">
         <is>
@@ -4950,8 +4968,10 @@
       <c r="X30" t="inlineStr"/>
       <c r="Y30" t="inlineStr"/>
       <c r="Z30" t="inlineStr"/>
-      <c r="AA30" t="n">
-        <v>9896659858</v>
+      <c r="AA30" t="inlineStr">
+        <is>
+          <t>9896659858</t>
+        </is>
       </c>
       <c r="AB30" t="inlineStr"/>
       <c r="AC30" t="inlineStr">
@@ -5111,8 +5131,10 @@
       </c>
       <c r="Y31" t="inlineStr"/>
       <c r="Z31" t="inlineStr"/>
-      <c r="AA31" t="n">
-        <v>8678198733</v>
+      <c r="AA31" t="inlineStr">
+        <is>
+          <t>8678198733</t>
+        </is>
       </c>
       <c r="AB31" t="inlineStr">
         <is>
@@ -5284,8 +5306,10 @@
       </c>
       <c r="Y32" t="inlineStr"/>
       <c r="Z32" t="inlineStr"/>
-      <c r="AA32" t="n">
-        <v>85987654689</v>
+      <c r="AA32" t="inlineStr">
+        <is>
+          <t>85987654689</t>
+        </is>
       </c>
       <c r="AB32" t="inlineStr">
         <is>
@@ -5699,8 +5723,10 @@
       <c r="X35" t="inlineStr"/>
       <c r="Y35" t="inlineStr"/>
       <c r="Z35" t="inlineStr"/>
-      <c r="AA35" t="n">
-        <v>8898654682</v>
+      <c r="AA35" t="inlineStr">
+        <is>
+          <t>8898654682</t>
+        </is>
       </c>
       <c r="AB35" t="inlineStr"/>
       <c r="AC35" t="inlineStr"/>
@@ -5751,6 +5777,812 @@
       <c r="AZ35" t="inlineStr"/>
       <c r="BA35" t="inlineStr"/>
     </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>79</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>HOSPITAL CLINICO SAO MATEUS</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>MAMÓGRAFO DIGITAL GE SENOGRAPHE CRYSTAL</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>ANTONIO</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>UNIDADE HOSPITALAR</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>[ALERTA FINANCEIRO: R$ 4,500.00 EM ABERTO] [CHAMADO ABERTO] MANUTENÇÃO PREVENTIVA PROGRAMADA E LIMPEZA GERAL</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+      <c r="T36" t="inlineStr"/>
+      <c r="U36" t="inlineStr"/>
+      <c r="V36" t="inlineStr"/>
+      <c r="W36" t="inlineStr"/>
+      <c r="X36" t="inlineStr">
+        <is>
+          <t>07.123.456/0001-99</t>
+        </is>
+      </c>
+      <c r="Y36" t="inlineStr"/>
+      <c r="Z36" t="inlineStr"/>
+      <c r="AA36" t="inlineStr"/>
+      <c r="AB36" t="inlineStr"/>
+      <c r="AC36" t="inlineStr"/>
+      <c r="AD36" t="inlineStr">
+        <is>
+          <t>SUGESTÃO: PREVENTIVA LIMPEZA &amp; LUBRIFICAÇÃO HOSPITALAR</t>
+        </is>
+      </c>
+      <c r="AE36" t="inlineStr"/>
+      <c r="AF36" t="inlineStr"/>
+      <c r="AG36" t="inlineStr"/>
+      <c r="AH36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI36" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO PREVENTIVA PROGRAMADA E LIMPEZA GERAL</t>
+        </is>
+      </c>
+      <c r="AJ36" t="inlineStr">
+        <is>
+          <t>OPERANDO COM FALHA</t>
+        </is>
+      </c>
+      <c r="AK36" t="inlineStr"/>
+      <c r="AL36" t="inlineStr"/>
+      <c r="AM36" t="inlineStr"/>
+      <c r="AN36" t="inlineStr"/>
+      <c r="AO36" t="inlineStr"/>
+      <c r="AP36" t="inlineStr">
+        <is>
+          <t>LIBERADO PARA USO NORMAL</t>
+        </is>
+      </c>
+      <c r="AQ36" t="inlineStr"/>
+      <c r="AR36" t="inlineStr"/>
+      <c r="AS36" t="inlineStr"/>
+      <c r="AT36" t="inlineStr"/>
+      <c r="AU36" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV36" t="inlineStr"/>
+      <c r="AW36" t="inlineStr"/>
+      <c r="AX36" t="inlineStr"/>
+      <c r="AY36" t="inlineStr"/>
+      <c r="AZ36" t="inlineStr"/>
+      <c r="BA36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>80</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>HOSPITAL CLINICO SAO MATEUS</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>RAIO-X DIGITAL SHIMADZU MOBILEDART</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>A DEFINIR / TRIAGEM PENDENTE</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>UNIDADE HOSPITALAR</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>[ALERTA FINANCEIRO: R$ 4,500.00 EM ABERTO] [CHAMADO ABERTO] SUBSTITUIÇÃO DO COLIMADOR E FALHA NO CAMPO LUMINOSO</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+      <c r="T37" t="inlineStr"/>
+      <c r="U37" t="inlineStr"/>
+      <c r="V37" t="inlineStr"/>
+      <c r="W37" t="inlineStr"/>
+      <c r="X37" t="inlineStr">
+        <is>
+          <t>07.123.456/0001-99</t>
+        </is>
+      </c>
+      <c r="Y37" t="inlineStr"/>
+      <c r="Z37" t="inlineStr"/>
+      <c r="AA37" t="inlineStr"/>
+      <c r="AB37" t="inlineStr"/>
+      <c r="AC37" t="inlineStr"/>
+      <c r="AD37" t="inlineStr">
+        <is>
+          <t>SUGESTÃO: SUBSTITUIÇÃO DE COLIMADOR &amp; ALINHAMENTO ÓPTICO (FEIXE R/X)</t>
+        </is>
+      </c>
+      <c r="AE37" t="inlineStr"/>
+      <c r="AF37" t="inlineStr"/>
+      <c r="AG37" t="inlineStr"/>
+      <c r="AH37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI37" t="inlineStr">
+        <is>
+          <t>SUBSTITUIÇÃO DO COLIMADOR E FALHA NO CAMPO LUMINOSO</t>
+        </is>
+      </c>
+      <c r="AJ37" t="inlineStr">
+        <is>
+          <t>OPERANDO COM FALHA</t>
+        </is>
+      </c>
+      <c r="AK37" t="inlineStr"/>
+      <c r="AL37" t="inlineStr"/>
+      <c r="AM37" t="inlineStr"/>
+      <c r="AN37" t="inlineStr"/>
+      <c r="AO37" t="inlineStr"/>
+      <c r="AP37" t="inlineStr">
+        <is>
+          <t>LIBERADO PARA USO NORMAL</t>
+        </is>
+      </c>
+      <c r="AQ37" t="inlineStr"/>
+      <c r="AR37" t="inlineStr"/>
+      <c r="AS37" t="inlineStr"/>
+      <c r="AT37" t="inlineStr"/>
+      <c r="AU37" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV37" t="inlineStr"/>
+      <c r="AW37" t="inlineStr"/>
+      <c r="AX37" t="inlineStr"/>
+      <c r="AY37" t="inlineStr"/>
+      <c r="AZ37" t="inlineStr"/>
+      <c r="BA37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>81</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>HOSPITAL CLINICO SAO MATEUS</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>MAMÓGRAFO DIGITAL GE SENOGRAPHE CRYSTAL</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>PREVENTIVA</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>ANTONIO</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>UNIDADE HOSPITALAR</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>[ALERTA FINANCEIRO: R$ 9,000.00 EM ABERTO] [CHAMADO ABERTO] MANUTENÇÃO PREVENTIVA PROGRAMADA E LIMPEZA GERAL</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+      <c r="T38" t="inlineStr"/>
+      <c r="U38" t="inlineStr"/>
+      <c r="V38" t="inlineStr"/>
+      <c r="W38" t="inlineStr"/>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>07.123.456/0001-99</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr"/>
+      <c r="Z38" t="inlineStr"/>
+      <c r="AA38" t="inlineStr"/>
+      <c r="AB38" t="inlineStr"/>
+      <c r="AC38" t="inlineStr"/>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>SUGESTÃO: PREVENTIVA LIMPEZA &amp; LUBRIFICAÇÃO HOSPITALAR</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr"/>
+      <c r="AF38" t="inlineStr"/>
+      <c r="AG38" t="inlineStr"/>
+      <c r="AH38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI38" t="inlineStr">
+        <is>
+          <t>MANUTENÇÃO PREVENTIVA PROGRAMADA E LIMPEZA GERAL</t>
+        </is>
+      </c>
+      <c r="AJ38" t="inlineStr">
+        <is>
+          <t>OPERANDO COM FALHA</t>
+        </is>
+      </c>
+      <c r="AK38" t="inlineStr"/>
+      <c r="AL38" t="inlineStr"/>
+      <c r="AM38" t="inlineStr"/>
+      <c r="AN38" t="inlineStr"/>
+      <c r="AO38" t="inlineStr"/>
+      <c r="AP38" t="inlineStr">
+        <is>
+          <t>LIBERADO PARA USO NORMAL</t>
+        </is>
+      </c>
+      <c r="AQ38" t="inlineStr"/>
+      <c r="AR38" t="inlineStr"/>
+      <c r="AS38" t="inlineStr"/>
+      <c r="AT38" t="inlineStr"/>
+      <c r="AU38" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV38" t="inlineStr"/>
+      <c r="AW38" t="inlineStr"/>
+      <c r="AX38" t="inlineStr"/>
+      <c r="AY38" t="inlineStr"/>
+      <c r="AZ38" t="inlineStr"/>
+      <c r="BA38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>82</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HOSPITAL CLINICO SAO MATEUS</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>RAIO-X DIGITAL SHIMADZU MOBILEDART</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>MARCOS</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>UNIDADE HOSPITALAR</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>[ALERTA FINANCEIRO: R$ 9,000.00 EM ABERTO] [CHAMADO ABERTO] SUBSTITUIÇÃO DO COLIMADOR E FALHA NO CAMPO LUMINOSO</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+      <c r="T39" t="inlineStr"/>
+      <c r="U39" t="inlineStr"/>
+      <c r="V39" t="inlineStr"/>
+      <c r="W39" t="inlineStr"/>
+      <c r="X39" t="inlineStr">
+        <is>
+          <t>07.123.456/0001-99</t>
+        </is>
+      </c>
+      <c r="Y39" t="inlineStr"/>
+      <c r="Z39" t="inlineStr"/>
+      <c r="AA39" t="inlineStr"/>
+      <c r="AB39" t="inlineStr"/>
+      <c r="AC39" t="inlineStr"/>
+      <c r="AD39" t="inlineStr">
+        <is>
+          <t>SUGESTÃO: SUBSTITUIÇÃO DE COLIMADOR &amp; ALINHAMENTO ÓPTICO (FEIXE R/X)</t>
+        </is>
+      </c>
+      <c r="AE39" t="inlineStr"/>
+      <c r="AF39" t="inlineStr"/>
+      <c r="AG39" t="inlineStr"/>
+      <c r="AH39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI39" t="inlineStr">
+        <is>
+          <t>SUBSTITUIÇÃO DO COLIMADOR E FALHA NO CAMPO LUMINOSO</t>
+        </is>
+      </c>
+      <c r="AJ39" t="inlineStr">
+        <is>
+          <t>OPERANDO COM FALHA</t>
+        </is>
+      </c>
+      <c r="AK39" t="inlineStr"/>
+      <c r="AL39" t="inlineStr"/>
+      <c r="AM39" t="inlineStr"/>
+      <c r="AN39" t="inlineStr"/>
+      <c r="AO39" t="inlineStr"/>
+      <c r="AP39" t="inlineStr">
+        <is>
+          <t>LIBERADO PARA USO NORMAL</t>
+        </is>
+      </c>
+      <c r="AQ39" t="inlineStr"/>
+      <c r="AR39" t="inlineStr"/>
+      <c r="AS39" t="inlineStr"/>
+      <c r="AT39" t="inlineStr"/>
+      <c r="AU39" t="inlineStr">
+        <is>
+          <t>NENHUM</t>
+        </is>
+      </c>
+      <c r="AV39" t="inlineStr"/>
+      <c r="AW39" t="inlineStr"/>
+      <c r="AX39" t="inlineStr"/>
+      <c r="AY39" t="inlineStr"/>
+      <c r="AZ39" t="inlineStr"/>
+      <c r="BA39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>83</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>HOSPITAL CLINICO SAO MATEUS</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>RAIO-X DIGITAL SHIMADZU MOBILEDART</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>A DEFINIR / TRIAGEM PENDENTE</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>UNIDADE HOSPITALAR</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>[CHAMADO ABERTO] SUBSTITUIÇÃO DO COLIMADOR E AJUSTE DE CAMPO</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>ATIVO</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
+      <c r="T40" t="inlineStr"/>
+      <c r="U40" t="inlineStr"/>
+      <c r="V40" t="inlineStr"/>
+      <c r="W40" t="inlineStr"/>
+      <c r="X40" t="inlineStr">
+        <is>
+          <t>07.123.456/0001-99</t>
+        </is>
+      </c>
+      <c r="Y40" t="inlineStr"/>
+      <c r="Z40" t="inlineStr"/>
+      <c r="AA40" t="inlineStr"/>
+      <c r="AB40" t="inlineStr"/>
+      <c r="AC40" t="inlineStr"/>
+      <c r="AD40" t="inlineStr">
+        <is>
+          <t>[SUGESTÃO: SUBSTITUIÇÃO DE COLIMADOR &amp; ALINHAMENTO ÓPTICO (FEIXE R/X)] FER-017: Kit de Alinhamento Óptico &amp; Centralização de Feixe R/X (Beam Alignment Tools) [✅ DISPONÍVEL NO ALMOXARIFADO] | FER-008: Nível Digital de Precisão e Trena Laser Métrica [✅ DISPONÍVEL NO ALMOXARIFADO] | FER-010: Torquímetro Calibrado com Jogo de Chaves Hexagonais / Torx [⏳ EM CAMPO COM ARQUIMEDES (AGUARDANDO RETORNO)] | PEC-015: Lâmpada Halógena de Colimador 12V/24V Sobressalente [⚠️ SEM SALDO (AGUARDANDO COMPRA/ENCOMENDA)] | CON-004: Panos de Microfibra ESD e Álcool Isopropílico 99% [✅ DISPONÍVEL (INSUMO / CONSUMÍVEL)]</t>
+        </is>
+      </c>
+      <c r="AE40" t="inlineStr"/>
+      <c r="AF40" t="inlineStr"/>
+      <c r="AG40" t="inlineStr"/>
+      <c r="AH40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI40" t="inlineStr">
+        <is>
+          <t>SUBSTITUIÇÃO DO COLIMADOR E AJUSTE DE CAMPO</t>
+        </is>
+      </c>
+      <c r="AJ40" t="inlineStr">
+        <is>
+          <t>OPERANDO COM FALHA</t>
+        </is>
+      </c>
+      <c r="AK40" t="inlineStr"/>
+      <c r="AL40" t="inlineStr"/>
+      <c r="AM40" t="inlineStr"/>
+      <c r="AN40" t="inlineStr"/>
+      <c r="AO40" t="inlineStr"/>
+      <c r="AP40" t="inlineStr">
+        <is>
+          <t>LIBERADO PARA USO NORMAL</t>
+        </is>
+      </c>
+      <c r="AQ40" t="inlineStr"/>
+      <c r="AR40" t="inlineStr"/>
+      <c r="AS40" t="inlineStr"/>
+      <c r="AT40" t="inlineStr"/>
+      <c r="AU40" t="inlineStr">
+        <is>
+          <t>NENHUM (INDIVIDUAL)</t>
+        </is>
+      </c>
+      <c r="AV40" t="inlineStr"/>
+      <c r="AW40" t="inlineStr"/>
+      <c r="AX40" t="inlineStr"/>
+      <c r="AY40" t="inlineStr"/>
+      <c r="AZ40" t="inlineStr"/>
+      <c r="BA40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>84</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HOSPITAL CLINICO SAO MATEUS</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>FORTALEZA</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>CE</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>RAIO-X DIGITAL SHIMADZU MOBILEDART</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>CORRETIVA</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>ARQUIMEDES</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>SIM</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-10-28</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>UNIDADE HOSPITALAR</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>[CONCLUÍDO - GERAL] Sem pendências restantes.</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>CONCLUÍDO</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>28/10/2026 21:05</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>28/10/2026 21:05</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>0 min</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>POP PADRÃO CONCLUÍDO</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>RESPONSÁVEL LOCAL</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>Arquimedes - Técnico</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr"/>
+      <c r="W41" t="inlineStr"/>
+      <c r="X41" t="inlineStr">
+        <is>
+          <t>07.123.456/0001-99</t>
+        </is>
+      </c>
+      <c r="Y41" t="inlineStr"/>
+      <c r="Z41" t="inlineStr"/>
+      <c r="AA41" t="inlineStr"/>
+      <c r="AB41" t="inlineStr"/>
+      <c r="AC41" t="inlineStr"/>
+      <c r="AD41" t="inlineStr"/>
+      <c r="AE41" t="inlineStr">
+        <is>
+          <t>GERAL</t>
+        </is>
+      </c>
+      <c r="AF41" t="inlineStr"/>
+      <c r="AG41" t="inlineStr">
+        <is>
+          <t>FATURAMENTO BOLETO BANCÁRIO — VALOR FINAL: R$ 450.00</t>
+        </is>
+      </c>
+      <c r="AH41" t="n">
+        <v>450</v>
+      </c>
+      <c r="AI41" t="inlineStr">
+        <is>
+          <t>SUBSTITUIÇÃO DO COLIMADOR E AJUSTE DE CAMPO</t>
+        </is>
+      </c>
+      <c r="AJ41" t="inlineStr">
+        <is>
+          <t>OPERANDO COM FALHA</t>
+        </is>
+      </c>
+      <c r="AK41" t="inlineStr"/>
+      <c r="AL41" t="inlineStr">
+        <is>
+          <t>DESGASTE NATURAL</t>
+        </is>
+      </c>
+      <c r="AM41" t="inlineStr">
+        <is>
+          <t>SUBSTITUIÇÃO DE COMPONENTE E REVISÃO GERAL DO COLIMADOR CONCLUÍDA. | [PEÇA JÁ CONTABILIZADA: 1x PEC-015 - LÂMPADA HALÓGENA DE COLIMADOR]</t>
+        </is>
+      </c>
+      <c r="AN41" t="inlineStr">
+        <is>
+          <t>DENTRO DAS NORMAS / HOMOLOGADO</t>
+        </is>
+      </c>
+      <c r="AO41" t="inlineStr"/>
+      <c r="AP41" t="inlineStr">
+        <is>
+          <t>LIBERADO PARA USO NORMAL</t>
+        </is>
+      </c>
+      <c r="AQ41" t="inlineStr"/>
+      <c r="AR41" t="inlineStr"/>
+      <c r="AS41" t="inlineStr"/>
+      <c r="AT41" t="inlineStr">
+        <is>
+          <t>1x PEC-015 - LÂMPADA HALÓGENA DE COLIMADOR</t>
+        </is>
+      </c>
+      <c r="AU41" t="inlineStr">
+        <is>
+          <t>NENHUM</t>
+        </is>
+      </c>
+      <c r="AV41" t="inlineStr"/>
+      <c r="AW41" t="inlineStr"/>
+      <c r="AX41" t="inlineStr"/>
+      <c r="AY41" t="inlineStr"/>
+      <c r="AZ41" t="inlineStr"/>
+      <c r="BA41" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(v38): fechamento contabil e levantamento de impostos, cotacao de transporte pesado/munck e cancelamento de notas com previa e leitor
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -2160,13 +2160,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>GABRIEL</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr"/>
+          <t>LEONARDO</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>558590000000</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2205,7 +2209,11 @@
           <t>CONTRATO</t>
         </is>
       </c>
-      <c r="AD12" t="inlineStr"/>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>SUGESTÃO: MANUTENÇÃO PREVENTIVA PADRÃO (RAIO-X / MAMOGRAFIA / ARCO)</t>
+        </is>
+      </c>
       <c r="AE12" t="inlineStr"/>
       <c r="AF12" t="inlineStr"/>
       <c r="AG12" t="inlineStr"/>
@@ -2278,10 +2286,14 @@
           <t>LEONARDO</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>558590000000</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -2320,7 +2332,11 @@
           <t>CONTRATO</t>
         </is>
       </c>
-      <c r="AD13" t="inlineStr"/>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>SUGESTÃO: MANUTENÇÃO PREVENTIVA PADRÃO (RAIO-X / MAMOGRAFIA / ARCO)</t>
+        </is>
+      </c>
       <c r="AE13" t="inlineStr"/>
       <c r="AF13" t="inlineStr"/>
       <c r="AG13" t="inlineStr"/>
@@ -2390,13 +2406,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>YASMIM</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr"/>
+          <t>LEONARDO</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>558590000000</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>NAO</t>
+          <t>SIM</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -2435,7 +2455,11 @@
           <t>CONTRATO</t>
         </is>
       </c>
-      <c r="AD14" t="inlineStr"/>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>SUGESTÃO: MANUTENÇÃO PREVENTIVA PADRÃO (RAIO-X / MAMOGRAFIA / ARCO)</t>
+        </is>
+      </c>
       <c r="AE14" t="inlineStr"/>
       <c r="AF14" t="inlineStr"/>
       <c r="AG14" t="inlineStr"/>
@@ -4389,12 +4413,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>EQUIPE EMED PLANTÃO</t>
+          <t>LEONARDO</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>(85) 3254-2929</t>
+          <t>558590000000</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -4480,7 +4504,7 @@
       </c>
       <c r="AD27" t="inlineStr">
         <is>
-          <t>SUGESTÃO: CALIBRAÇÃO &amp; MANUTENÇÃO EM DENSITOMETRIA ÓSSEA</t>
+          <t>SUGESTÃO GERAL DE ATENDIMENTO</t>
         </is>
       </c>
       <c r="AE27" t="inlineStr">
@@ -4521,11 +4545,7 @@
       <c r="AR27" t="inlineStr"/>
       <c r="AS27" t="inlineStr"/>
       <c r="AT27" t="inlineStr"/>
-      <c r="AU27" t="inlineStr">
-        <is>
-          <t>NENHUM (INDIVIDUAL)</t>
-        </is>
-      </c>
+      <c r="AU27" t="inlineStr"/>
       <c r="AV27" t="inlineStr"/>
       <c r="AW27" t="inlineStr"/>
       <c r="AX27" t="inlineStr"/>
@@ -5808,10 +5828,14 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>ANTONIO</t>
-        </is>
-      </c>
-      <c r="H36" t="inlineStr"/>
+          <t>MARCOS</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>8599912312124</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -5859,7 +5883,7 @@
       <c r="AC36" t="inlineStr"/>
       <c r="AD36" t="inlineStr">
         <is>
-          <t>SUGESTÃO: PREVENTIVA LIMPEZA &amp; LUBRIFICAÇÃO HOSPITALAR</t>
+          <t>SUGESTÃO: MANUTENÇÃO PREVENTIVA PADRÃO (RAIO-X / MAMOGRAFIA / ARCO)</t>
         </is>
       </c>
       <c r="AE36" t="inlineStr"/>
@@ -5892,11 +5916,7 @@
       <c r="AR36" t="inlineStr"/>
       <c r="AS36" t="inlineStr"/>
       <c r="AT36" t="inlineStr"/>
-      <c r="AU36" t="inlineStr">
-        <is>
-          <t>NENHUM (INDIVIDUAL)</t>
-        </is>
-      </c>
+      <c r="AU36" t="inlineStr"/>
       <c r="AV36" t="inlineStr"/>
       <c r="AW36" t="inlineStr"/>
       <c r="AX36" t="inlineStr"/>
@@ -5935,10 +5955,14 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>A DEFINIR / TRIAGEM PENDENTE</t>
-        </is>
-      </c>
-      <c r="H37" t="inlineStr"/>
+          <t>MARCOS</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>8599912312124</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -6019,11 +6043,7 @@
       <c r="AR37" t="inlineStr"/>
       <c r="AS37" t="inlineStr"/>
       <c r="AT37" t="inlineStr"/>
-      <c r="AU37" t="inlineStr">
-        <is>
-          <t>NENHUM (INDIVIDUAL)</t>
-        </is>
-      </c>
+      <c r="AU37" t="inlineStr"/>
       <c r="AV37" t="inlineStr"/>
       <c r="AW37" t="inlineStr"/>
       <c r="AX37" t="inlineStr"/>
@@ -6062,10 +6082,14 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>ANTONIO</t>
-        </is>
-      </c>
-      <c r="H38" t="inlineStr"/>
+          <t>MARCOS</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>8599912312124</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -6113,7 +6137,7 @@
       <c r="AC38" t="inlineStr"/>
       <c r="AD38" t="inlineStr">
         <is>
-          <t>SUGESTÃO: PREVENTIVA LIMPEZA &amp; LUBRIFICAÇÃO HOSPITALAR</t>
+          <t>SUGESTÃO: MANUTENÇÃO PREVENTIVA PADRÃO (RAIO-X / MAMOGRAFIA / ARCO)</t>
         </is>
       </c>
       <c r="AE38" t="inlineStr"/>
@@ -6146,11 +6170,7 @@
       <c r="AR38" t="inlineStr"/>
       <c r="AS38" t="inlineStr"/>
       <c r="AT38" t="inlineStr"/>
-      <c r="AU38" t="inlineStr">
-        <is>
-          <t>NENHUM (INDIVIDUAL)</t>
-        </is>
-      </c>
+      <c r="AU38" t="inlineStr"/>
       <c r="AV38" t="inlineStr"/>
       <c r="AW38" t="inlineStr"/>
       <c r="AX38" t="inlineStr"/>
@@ -6192,7 +6212,11 @@
           <t>MARCOS</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr"/>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>8599912312124</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -6273,11 +6297,7 @@
       <c r="AR39" t="inlineStr"/>
       <c r="AS39" t="inlineStr"/>
       <c r="AT39" t="inlineStr"/>
-      <c r="AU39" t="inlineStr">
-        <is>
-          <t>NENHUM</t>
-        </is>
-      </c>
+      <c r="AU39" t="inlineStr"/>
       <c r="AV39" t="inlineStr"/>
       <c r="AW39" t="inlineStr"/>
       <c r="AX39" t="inlineStr"/>
@@ -6316,10 +6336,14 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>A DEFINIR / TRIAGEM PENDENTE</t>
-        </is>
-      </c>
-      <c r="H40" t="inlineStr"/>
+          <t>MARCOS</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>8599912312124</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>SIM</t>
@@ -6367,7 +6391,7 @@
       <c r="AC40" t="inlineStr"/>
       <c r="AD40" t="inlineStr">
         <is>
-          <t>[SUGESTÃO: SUBSTITUIÇÃO DE COLIMADOR &amp; ALINHAMENTO ÓPTICO (FEIXE R/X)] FER-017: Kit de Alinhamento Óptico &amp; Centralização de Feixe R/X (Beam Alignment Tools) [✅ DISPONÍVEL NO ALMOXARIFADO] | FER-008: Nível Digital de Precisão e Trena Laser Métrica [✅ DISPONÍVEL NO ALMOXARIFADO] | FER-010: Torquímetro Calibrado com Jogo de Chaves Hexagonais / Torx [⏳ EM CAMPO COM ARQUIMEDES (AGUARDANDO RETORNO)] | PEC-015: Lâmpada Halógena de Colimador 12V/24V Sobressalente [⚠️ SEM SALDO (AGUARDANDO COMPRA/ENCOMENDA)] | CON-004: Panos de Microfibra ESD e Álcool Isopropílico 99% [✅ DISPONÍVEL (INSUMO / CONSUMÍVEL)]</t>
+          <t>SUGESTÃO: SUBSTITUIÇÃO DE COLIMADOR &amp; ALINHAMENTO ÓPTICO (FEIXE R/X)</t>
         </is>
       </c>
       <c r="AE40" t="inlineStr"/>
@@ -6400,11 +6424,7 @@
       <c r="AR40" t="inlineStr"/>
       <c r="AS40" t="inlineStr"/>
       <c r="AT40" t="inlineStr"/>
-      <c r="AU40" t="inlineStr">
-        <is>
-          <t>NENHUM (INDIVIDUAL)</t>
-        </is>
-      </c>
+      <c r="AU40" t="inlineStr"/>
       <c r="AV40" t="inlineStr"/>
       <c r="AW40" t="inlineStr"/>
       <c r="AX40" t="inlineStr"/>

</xml_diff>

<commit_message>
fix(dados): consolidar restauracao da base operacional limpa de clientes e OSs
</commit_message>
<xml_diff>
--- a/base_clientes.xlsx
+++ b/base_clientes.xlsx
@@ -6385,7 +6385,11 @@
         </is>
       </c>
       <c r="Y40" t="inlineStr"/>
-      <c r="Z40" t="inlineStr"/>
+      <c r="Z40" t="inlineStr">
+        <is>
+          <t>financeiro@saomateus.com.br</t>
+        </is>
+      </c>
       <c r="AA40" t="inlineStr"/>
       <c r="AB40" t="inlineStr"/>
       <c r="AC40" t="inlineStr"/>

</xml_diff>